<commit_message>
feat: delete task (DELETE /api/tasks/:id) and jump-to-project-folder button (POST /api/fs/open)
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G53"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -620,27 +620,27 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="0">
         <is>
-          <t>列标题图标</t>
+          <t>直达项目目录</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="0">
         <is>
-          <t>看四个列标题前的圆圈</t>
+          <t>点任意卡片标题旁的 📁 按钮</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="0">
         <is>
-          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
+          <t>服务器那台电脑弹出资源管理器/访达，定位到该任务的 workspace 文件夹；路径不存在时提示错误</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="0">
@@ -657,7 +657,7 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
@@ -667,17 +667,17 @@
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t>无整条色带</t>
+          <t>列标题图标</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t>看列头背景</t>
+          <t>看四个列标题前的圆圈</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>列头是白底细边，不是一整条颜色</t>
+          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
@@ -694,27 +694,27 @@
     <row r="18">
       <c r="A18" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 四列看板</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t>接取按钮默认隐藏</t>
+          <t>无整条色带</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>未保存 agent 身份时看待处理卡片</t>
+          <t>看列头背景</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>卡片上**没有**「接取」按钮（agent 通过 API 自己接取）</t>
+          <t>列头是白底细边，不是一整条颜色</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
@@ -731,7 +731,7 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
@@ -741,17 +741,17 @@
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>保存身份后按钮出现</t>
+          <t>接取按钮默认隐藏</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t>Agent 管理填 agentId + 名称 →「保存身份」→ 看待处理卡片</t>
+          <t>未保存 agent 身份时看待处理卡片</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>出现「接取」按钮</t>
+          <t>卡片上**没有**「接取」按钮（agent 通过 API 自己接取）</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
@@ -768,7 +768,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
@@ -778,17 +778,17 @@
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>正常接取</t>
+          <t>保存身份后按钮出现</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>点「接取」</t>
+          <t>Agent 管理填 agentId + 名称 →「保存身份」→ 看待处理卡片</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**处理中**列（黄圈），标题旁显示头像或彩色圆+首字母</t>
+          <t>出现「接取」按钮</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,7 +805,7 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
@@ -815,17 +815,17 @@
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>图片头像</t>
+          <t>正常接取</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>身份表单选一张图片 → 保存 → 接取</t>
+          <t>点「接取」</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>卡片标题旁显示该图片（圆形裁剪），Agent 列表里也有</t>
+          <t>卡片移到**处理中**列（黄圈），标题旁显示头像或彩色圆+首字母</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,7 +842,7 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
@@ -852,17 +852,17 @@
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>无头像接取</t>
+          <t>图片头像</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>不选图片保存身份后接取</t>
+          <t>身份表单选一张图片 → 保存 → 接取</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>显示彩色圆（颜色随名字变化）+ 名字首字母</t>
+          <t>卡片标题旁显示该图片（圆形裁剪），Agent 列表里也有</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,7 +879,7 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
@@ -889,17 +889,17 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>多个 agent</t>
+          <t>无头像接取</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>换一个 agentId 接取另一个任务</t>
+          <t>不选图片保存身份后接取</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>每个卡片显示各自的 agent 头像</t>
+          <t>显示彩色圆（颜色随名字变化）+ 名字首字母</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,7 +916,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
@@ -926,17 +926,17 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>多个 agent</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>两个身份先后点同一个「接取」（或开两个浏览器窗口同时点）</t>
+          <t>换一个 agentId 接取另一个任务</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>**只有一个人成功**，另一个弹「task is not in the required status for claim」</t>
+          <t>每个卡片显示各自的 agent 头像</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,27 +953,27 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
         <is>
-          <t>E. 阻碍 / 解除阻碍 / 完成</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>阻碍</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>处理中的卡片点「阻碍」</t>
+          <t>两个身份先后点同一个「接取」（或开两个浏览器窗口同时点）</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**遇到阻碍**列（红 ! 圈）</t>
+          <t>**只有一个人成功**，另一个弹「task is not in the required status for claim」</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,7 +990,7 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
@@ -1000,17 +1000,17 @@
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>解除阻碍</t>
+          <t>阻碍</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>遇到阻碍的卡片点「解除阻碍」</t>
+          <t>处理中的卡片点「阻碍」</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**处理中**列，仍是原 agent</t>
+          <t>卡片移到**遇到阻碍**列（红 ! 圈）</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,7 +1027,7 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>E3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>完成</t>
+          <t>解除阻碍</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>处理中的卡片点「完成」</t>
+          <t>遇到阻碍的卡片点「解除阻碍」</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**等你确认**列（绿 ✓ 圈）</t>
+          <t>卡片回到**处理中**列，仍是原 agent</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,7 +1064,7 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>E4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>错误状态操作</t>
+          <t>完成</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>对**待处理**的卡片点「完成」</t>
+          <t>处理中的卡片点「完成」</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>弹操作失败（conflict 提示），卡片不动</t>
+          <t>卡片移到**等你确认**列（绿 ✓ 圈）</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,27 +1101,27 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 阻碍 / 解除阻碍 / 完成</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>错误状态操作</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>等你确认的卡片点「验收通过（归档）」</t>
+          <t>对**待处理**的卡片点「完成」</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；点右上「归档历史」能看到它，带「完成于 …」时间</t>
+          <t>弹操作失败（conflict 提示），卡片不动</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,7 +1138,7 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
@@ -1148,17 +1148,17 @@
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>退回修改</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>另一张等你确认的卡片点「退回修改」</t>
+          <t>等你确认的卡片点「验收通过（归档）」</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**处理中**列，仍是原 agent</t>
+          <t>卡片从四列消失；点右上「归档历史」能看到它，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,7 +1175,7 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>退回修改</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>归档历史里看卡片</t>
+          <t>另一张等你确认的卡片点「退回修改」</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>显示标题、类型、标签、完成时间</t>
+          <t>卡片回到**处理中**列，仍是原 agent</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,7 +1212,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>历史收起</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>再点「归档历史」</t>
+          <t>归档历史里看卡片</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>历史区隐藏，按钮文字变回「归档历史」</t>
+          <t>显示标题、类型、标签、完成时间</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,27 +1249,27 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>编辑字段</t>
+          <t>历史收起</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「编辑」→ 改标题/描述/类型/标签 → 保存</t>
+          <t>再点「归档历史」</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>卡片内容更新</t>
+          <t>历史区隐藏，按钮文字变回「归档历史」</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,7 +1286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1296,17 +1296,17 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>编辑字段</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
+          <t>任意卡片点「编辑」→ 改标题/描述/类型/标签 → 保存</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>卡片内容更新</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,7 +1323,7 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
@@ -1333,17 +1333,17 @@
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>编辑里把类型清空、标签清空 → 保存</t>
+          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>卡片上的类型徽章和标签消失</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,7 +1360,7 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
@@ -1370,17 +1370,17 @@
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>编辑已归档任务</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>历史里没有编辑入口</t>
+          <t>编辑里把类型清空、标签清空 → 保存</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>归档历史只读（符合预期）</t>
+          <t>卡片上的类型徽章和标签消失</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,27 +1397,27 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 管理</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>Agent 管理填 id + 名称，头像选一张图片 → 「预配置 / 更新」</t>
+          <t>任意卡片点「删除」→ 确认弹窗</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>下方列表出现该 agent，显示图片头像</t>
+          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,27 +1434,27 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 管理</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>编辑已归档任务</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>再次提交同一 id、换一张图片</t>
+          <t>历史里没有编辑入口</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>列表里头像更新；之后它接取的卡片显示新头像</t>
+          <t>归档历史只读（符合预期）</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,7 +1471,7 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>空名称预配置</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>只填 id 提交</t>
+          <t>Agent 管理填 id + 名称，头像选一张图片 → 「预配置 / 更新」</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>自动以 id 作为名称</t>
+          <t>下方列表出现该 agent，显示图片头像</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,27 +1508,27 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 管理</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>回收</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「回收」</t>
+          <t>再次提交同一 id、换一张图片</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>列表里头像更新；之后它接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 管理</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>空名称预配置</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>只填 id 提交</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>自动以 id 作为名称</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,7 +1582,7 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>回收</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>处理中卡片点「回收」</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>卡片回到**待处理**列，agent 头像消失</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,27 +1619,27 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>回收后再点「接取」</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,27 +1656,27 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>疑似卡住标记</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,7 +1693,7 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
@@ -1703,17 +1703,17 @@
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,7 +1730,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,7 +1767,7 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
@@ -1777,17 +1777,17 @@
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>第一次 200，第二次 409 + error 信息</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,27 +1804,27 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>返回已归档任务数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,27 +1841,27 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,7 +1878,7 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
@@ -1888,17 +1888,17 @@
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>Gatekeeper</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>首次运行若提示"无法验证开发者"</t>
+          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,35 +1915,109 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr" s="0">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr" s="0">
+        <is>
+          <t>Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr" s="0">
+        <is>
+          <t>首次运行若提示"无法验证开发者"</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr" s="0">
+        <is>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr" s="0">
+        <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr" s="0">
+      <c r="B53" t="inlineStr" s="0">
         <is>
           <t>K. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr" s="0">
+      <c r="C53" t="inlineStr" s="0">
         <is>
           <t>系统选择</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr" s="0">
+      <c r="D53" t="inlineStr" s="0">
         <is>
           <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr" s="0">
+      <c r="E53" t="inlineStr" s="0">
         <is>
           <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr" s="0">
+      <c r="F53" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -1951,7 +2025,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F51">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F53">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: claim-time identity constraints — name and real image avatar required (no fabricated avatar paths); pin human-configured identities; clearer agent list
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -783,12 +783,12 @@
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>Agent 管理填 agentId + 名称 →「保存身份」→ 看待处理卡片</t>
+          <t>Agent 管理填 agentId + 名称 + 头像图片 →「保存身份」→ 看待处理卡片</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>出现「接取」按钮</t>
+          <t>出现「接取」按钮；缺名称或头像时保存被拒并提示</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -825,7 +825,7 @@
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**处理中**列（黄圈），标题旁显示头像或彩色圆+首字母</t>
+          <t>卡片移到**处理中**列（黄圈），标题旁显示图片头像 + 名称</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -889,17 +889,17 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>无头像接取</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>不选图片保存身份后接取</t>
+          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>显示彩色圆（颜色随名字变化）+ 名字首字母</t>
+          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -1582,27 +1582,27 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 管理</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>回收</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「回收」</t>
+          <t>预配置 id/名称/头像后，该 agent 用别的名字/头像接取</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>看板仍显示预配置的名称和头像（不被 agent 覆盖）</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,7 +1619,7 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
@@ -1629,17 +1629,17 @@
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>回收</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>处理中卡片点「回收」</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>卡片回到**待处理**列，agent 头像消失</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,7 +1656,7 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
@@ -1666,17 +1666,17 @@
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>回收后再点「接取」</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>疑似卡住标记</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,7 +1730,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,7 +1767,7 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
@@ -1777,17 +1777,17 @@
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,7 +1804,7 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
@@ -1814,17 +1814,17 @@
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>第一次 200，第二次 409 + error 信息</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,7 +1841,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>返回已归档任务数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,27 +1878,27 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,7 +1915,7 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,7 +1952,7 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>Gatekeeper</t>
+          <t>Intel Mac</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>首次运行若提示"无法验证开发者"</t>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,35 +1989,72 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr" s="0">
+        <is>
+          <t>Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr" s="0">
+        <is>
+          <t>首次运行若提示"无法验证开发者"</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr" s="0">
+        <is>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr" s="0">
+        <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr" s="0">
+      <c r="B54" t="inlineStr" s="0">
         <is>
           <t>K. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr" s="0">
+      <c r="C54" t="inlineStr" s="0">
         <is>
           <t>系统选择</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr" s="0">
+      <c r="D54" t="inlineStr" s="0">
         <is>
           <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr" s="0">
+      <c r="E54" t="inlineStr" s="0">
         <is>
           <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr" s="0">
+      <c r="F54" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2025,7 +2062,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F53">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F54">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
ui: add-task and archive-history become top-bar modals; remove type field (tags only); hide agent registration from UI (agents self-register via claim API, card shows avatar+name with id pill)
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G57"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -265,12 +265,12 @@
       </c>
       <c r="D6" t="inlineStr" s="0">
         <is>
-          <t>只填「任务标题」和「workspace 文件夹路径」，点「添加任务」</t>
+          <t>点右上「＋ 添加任务」→ 弹窗填「任务标题」和「workspace 文件夹路径」→ 点「添加」</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>任务出现在**待处理**列（灰圈图标）</t>
+          <t>弹窗关闭，任务出现在**待处理**列（灰圈图标）</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
@@ -302,7 +302,7 @@
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>只填路径，点添加</t>
+          <t>弹窗只填路径，点添加</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
@@ -339,7 +339,7 @@
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>只填标题，点添加</t>
+          <t>弹窗只填标题，点添加</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
@@ -376,12 +376,12 @@
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t>添加时填描述、类型、标签、截止时间</t>
+          <t>添加时填描述、标签、截止时间</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>卡片上显示绿色类型徽章、紫色标签、黄色「截止…」提示</t>
+          <t>卡片上显示紫色标签、黄色「截止…」提示、描述文本</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
@@ -408,17 +408,17 @@
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t>类型 vs 标签</t>
+          <t>多个标签</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t>类型填 `feature`，标签填 `go, ui`</t>
+          <t>标签填 `go, ui`</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>类型只有一个（feature），标签有两个（go、ui），样式不同</t>
+          <t>显示两个紫色标签</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
@@ -657,27 +657,27 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t>列标题图标</t>
+          <t>取消添加</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t>看四个列标题前的圆圈</t>
+          <t>点「＋ 添加任务」→ 点「取消」或点弹窗外区域</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
+          <t>弹窗关闭，没有任务被创建</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
@@ -694,7 +694,7 @@
     <row r="18">
       <c r="A18" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
@@ -704,17 +704,17 @@
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t>无整条色带</t>
+          <t>列标题图标</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>看列头背景</t>
+          <t>看四个列标题前的圆圈</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>列头是白底细边，不是一整条颜色</t>
+          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
@@ -731,27 +731,27 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 四列看板</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>接取按钮默认隐藏</t>
+          <t>无整条色带</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t>未保存 agent 身份时看待处理卡片</t>
+          <t>看列头背景</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>卡片上**没有**「接取」按钮（agent 通过 API 自己接取）</t>
+          <t>列头是白底细边，不是一整条颜色</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
@@ -768,7 +768,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
@@ -778,17 +778,17 @@
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>保存身份后按钮出现</t>
+          <t>主界面无注册入口</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>Agent 管理填 agentId + 名称 + 头像图片 →「保存身份」→ 看待处理卡片</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>出现「接取」按钮；缺名称或头像时保存被拒并提示</t>
+          <t>页面上**没有**「Agent 管理 / 注册」表单；agent 信息只出现在被它接取的卡片上</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,7 +805,7 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
@@ -815,17 +815,17 @@
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>正常接取</t>
+          <t>API 注册并接取</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>点「接取」</t>
+          <t>先上传头像：`curl -F "file=@头像.png" http://localhost:8080/api/avatars`，记下返回的 `path`；再 claim：`curl -X POST -H "Content-Type: application/json" -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;上一步的path&gt;"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**处理中**列（黄圈），标题旁显示图片头像 + 名称</t>
+          <t>返回 200，卡片移到**处理中**列，标题旁显示图片头像 + 名称</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,7 +842,7 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
@@ -852,17 +852,17 @@
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>图片头像</t>
+          <t>名称与 id 分开显示</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>身份表单选一张图片 → 保存 → 接取</t>
+          <t>用名称 `Grok Build`、id `grok build` 接取后看卡片</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>卡片标题旁显示该图片（圆形裁剪），Agent 列表里也有</t>
+          <t>卡片显示加粗名称「Grok Build」+ 灰色小药丸 id「grok build」，不会连成一串</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,7 +879,7 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
@@ -889,17 +889,17 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>缺名称/头像被拒</t>
+          <t>图片头像</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
+          <t>接取后看卡片</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
+          <t>显示上传的图片（圆形裁剪），不是字母/表情符号</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,7 +916,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
@@ -926,17 +926,17 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>多个 agent</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>换一个 agentId 接取另一个任务</t>
+          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>每个卡片显示各自的 agent 头像</t>
+          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,7 +953,7 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
@@ -963,17 +963,17 @@
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>多个 agent</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>两个身份先后点同一个「接取」（或开两个浏览器窗口同时点）</t>
+          <t>换一个 agentId 接取另一个任务</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>**只有一个人成功**，另一个弹「task is not in the required status for claim」</t>
+          <t>每个卡片显示各自的 agent 头像</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,27 +990,27 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t>E. 阻碍 / 解除阻碍 / 完成</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>阻碍</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>处理中的卡片点「阻碍」</t>
+          <t>两个不同 agentId 先后 claim 同一任务（或开两个浏览器窗口同时点）</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**遇到阻碍**列（红 ! 圈）</t>
+          <t>**只有一个人成功**，另一个 409 + 提示</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,7 +1027,7 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>解除阻碍</t>
+          <t>阻碍</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>遇到阻碍的卡片点「解除阻碍」</t>
+          <t>处理中的卡片点「阻碍」</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**处理中**列，仍是原 agent</t>
+          <t>卡片移到**遇到阻碍**列（红 ! 圈）</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,7 +1064,7 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>E3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>完成</t>
+          <t>解除阻碍</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>处理中的卡片点「完成」</t>
+          <t>遇到阻碍的卡片点「解除阻碍」</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**等你确认**列（绿 ✓ 圈）</t>
+          <t>卡片回到**处理中**列，仍是原 agent</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,7 +1101,7 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>E4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>错误状态操作</t>
+          <t>完成</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>对**待处理**的卡片点「完成」</t>
+          <t>处理中的卡片点「完成」</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>弹操作失败（conflict 提示），卡片不动</t>
+          <t>卡片移到**等你确认**列（绿 ✓ 圈）</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,27 +1138,27 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 阻碍 / 解除阻碍 / 完成</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>错误状态操作</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>等你确认的卡片点「验收通过（归档）」</t>
+          <t>对**待处理**的卡片点「完成」</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；点右上「归档历史」能看到它，带「完成于 …」时间</t>
+          <t>弹操作失败（conflict 提示），卡片不动</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,7 +1175,7 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>退回修改</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>另一张等你确认的卡片点「退回修改」</t>
+          <t>等你确认的卡片点「验收通过（归档）」</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**处理中**列，仍是原 agent</t>
+          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,7 +1212,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>退回修改</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>归档历史里看卡片</t>
+          <t>另一张等你确认的卡片点「退回修改」</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>显示标题、类型、标签、完成时间</t>
+          <t>卡片回到**处理中**列，仍是原 agent</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,7 +1249,7 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
@@ -1259,17 +1259,17 @@
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>历史收起</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>再点「归档历史」</t>
+          <t>归档历史弹窗里看条目</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>历史区隐藏，按钮文字变回「归档历史」</t>
+          <t>显示标题、标签、完成时间</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,27 +1286,27 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>编辑字段</t>
+          <t>历史关闭</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「编辑」→ 改标题/描述/类型/标签 → 保存</t>
+          <t>点「关闭」或点击弹窗外区域</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>卡片内容更新</t>
+          <t>弹窗关闭，看板恢复正常</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,27 +1323,27 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
+          <t>历史弹窗里点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>该条消失，看板和历史里都不再有</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,27 +1360,27 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>全选删除</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>编辑里把类型清空、标签清空 → 保存</t>
+          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>卡片上的类型徽章和标签消失</t>
+          <t>选中的条目全部消失</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,7 +1397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>编辑字段</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「删除」→ 确认弹窗</t>
+          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
+          <t>卡片内容更新</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,7 +1434,7 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>编辑已归档任务</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>历史里没有编辑入口</t>
+          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>归档历史只读（符合预期）</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,27 +1471,27 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 管理</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>Agent 管理填 id + 名称，头像选一张图片 → 「预配置 / 更新」</t>
+          <t>编辑里把标签清空 → 保存</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>下方列表出现该 agent，显示图片头像</t>
+          <t>卡片上的标签消失</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,27 +1508,27 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 管理</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>再次提交同一 id、换一张图片</t>
+          <t>任意卡片点「删除」→ 确认弹窗</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>列表里头像更新；之后它接取的卡片显示新头像</t>
+          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 管理</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>空名称预配置</t>
+          <t>编辑已归档任务</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>只填 id 提交</t>
+          <t>历史里没有编辑入口</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>自动以 id 作为名称</t>
+          <t>归档历史只读（符合预期）</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,27 +1582,27 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>H4</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 管理</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>预配置 id/名称/头像后，该 agent 用别的名字/头像接取</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>看板仍显示预配置的名称和头像（不被 agent 覆盖）</t>
+          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,27 +1619,27 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>回收</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「回收」</t>
+          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>之后该 agent 接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,27 +1656,27 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>空名称预配置</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>名称自动等于 id</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>预配置后，该 agent claim 时带别的名称/头像</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,27 +1730,27 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>回收</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>处理中卡片点「回收」</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>卡片回到**待处理**列，agent 头像消失</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,27 +1767,27 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>回收后再点「接取」</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,27 +1804,27 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>疑似卡住标记</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,7 +1841,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,7 +1878,7 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
@@ -1888,17 +1888,17 @@
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,27 +1915,27 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>第一次 200，第二次 409 + error 信息</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,27 +1952,27 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>返回已归档任务数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,27 +1989,27 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>Gatekeeper</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>首次运行若提示"无法验证开发者"</t>
+          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,35 +2026,146 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr" s="0">
+        <is>
+          <t>Apple Silicon</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr" s="0">
+        <is>
+          <t>正常启动，页面功能同 Windows</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr" s="0">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr" s="0">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr" s="0">
+        <is>
+          <t>Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr" s="0">
+        <is>
+          <t>首次运行若提示"无法验证开发者"</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr" s="0">
+        <is>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr" s="0">
+        <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr" s="0">
+      <c r="B57" t="inlineStr" s="0">
         <is>
           <t>K. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr" s="0">
+      <c r="C57" t="inlineStr" s="0">
         <is>
           <t>系统选择</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr" s="0">
+      <c r="D57" t="inlineStr" s="0">
         <is>
           <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr" s="0">
+      <c r="E57" t="inlineStr" s="0">
         <is>
           <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr" s="0">
+      <c r="F57" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2062,7 +2173,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F54">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F57">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
ui: card buttons are only human actions — edit/delete everywhere plus archive on awaiting confirmation; status transitions (block/unblock/complete/recycle/reject) are agent-API-only
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -852,7 +852,7 @@
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>名称与 id 分开显示</t>
+          <t>卡片只显示名称</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
@@ -862,7 +862,7 @@
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>卡片显示加粗名称「Grok Build」+ 灰色小药丸 id「grok build」，不会连成一串</t>
+          <t>卡片只显示图片头像 + 加粗名称「Grok Build」，**不显示** id（id 仅存在于 API 层）</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -1032,22 +1032,22 @@
       </c>
       <c r="B27" t="inlineStr" s="0">
         <is>
-          <t>E. 阻碍 / 解除阻碍 / 完成</t>
+          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>阻碍</t>
+          <t>处理中/阻碍卡片按钮</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>处理中的卡片点「阻碍」</t>
+          <t>看「处理中」「遇到阻碍」列的卡片</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**遇到阻碍**列（红 ! 圈）</t>
+          <t>只显示「编辑」「删除」，没有「阻碍/完成/回收/解除阻碍」按钮</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1069,22 +1069,22 @@
       </c>
       <c r="B28" t="inlineStr" s="0">
         <is>
-          <t>E. 阻碍 / 解除阻碍 / 完成</t>
+          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>解除阻碍</t>
+          <t>API 状态流转</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>遇到阻碍的卡片点「解除阻碍」</t>
+          <t>用 curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**处理中**列，仍是原 agent</t>
+          <t>卡片在列间正确移动（这是 agent 的动作，界面不提供按钮）</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,27 +1101,27 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>E3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
         <is>
-          <t>E. 阻碍 / 解除阻碍 / 完成</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>完成</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>处理中的卡片点「完成」</t>
+          <t>等你确认的卡片点「验收通过（归档）」</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>卡片移到**等你确认**列（绿 ✓ 圈）</t>
+          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,27 +1138,27 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>E4</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t>E. 阻碍 / 解除阻碍 / 完成</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>错误状态操作</t>
+          <t>无退回修改按钮</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>对**待处理**的卡片点「完成」</t>
+          <t>看「等你确认」卡片</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>弹操作失败（conflict 提示），卡片不动</t>
+          <t>只有「验收通过（归档）」「编辑」「删除」，没有「退回修改」——要退回时直接命令 agent，agent 自己调 API 把任务退回「处理中」</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,7 +1175,7 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>等你确认的卡片点「验收通过（归档）」</t>
+          <t>归档历史弹窗里看条目</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
+          <t>显示标题、标签、完成时间</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,7 +1212,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>退回修改</t>
+          <t>历史关闭</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>另一张等你确认的卡片点「退回修改」</t>
+          <t>点「关闭」或点击弹窗外区域</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**处理中**列，仍是原 agent</t>
+          <t>弹窗关闭，看板恢复正常</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,7 +1249,7 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
@@ -1259,17 +1259,17 @@
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>归档历史弹窗里看条目</t>
+          <t>历史弹窗里点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>显示标题、标签、完成时间</t>
+          <t>该条消失，看板和历史里都不再有</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,7 +1286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1296,17 +1296,17 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>历史关闭</t>
+          <t>全选删除</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>点「关闭」或点击弹窗外区域</t>
+          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，看板恢复正常</t>
+          <t>选中的条目全部消失</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,27 +1323,27 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>F5</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>单条删除</t>
+          <t>编辑字段</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗里点某条「删除」→ 确认</t>
+          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>该条消失，看板和历史里都不再有</t>
+          <t>卡片内容更新</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,27 +1360,27 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>F6</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>全选删除</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
+          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>选中的条目全部消失</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,7 +1397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>编辑字段</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
+          <t>编辑里把标签清空 → 保存</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>卡片内容更新</t>
+          <t>卡片上的标签消失</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,7 +1434,7 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
+          <t>任意卡片点「删除」→ 确认弹窗</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,7 +1471,7 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>编辑已归档任务</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>编辑里把标签清空 → 保存</t>
+          <t>历史里没有编辑入口</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>卡片上的标签消失</t>
+          <t>归档历史只读（符合预期）</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,27 +1508,27 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「删除」→ 确认弹窗</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
+          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>G5</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>编辑已归档任务</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>历史里没有编辑入口</t>
+          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>归档历史只读（符合预期）</t>
+          <t>之后该 agent 接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,7 +1582,7 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>空名称预配置</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
+          <t>名称自动等于 id</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,7 +1619,7 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
@@ -1629,17 +1629,17 @@
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
+          <t>预配置后，该 agent claim 时带别的名称/头像</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>之后该 agent 接取的卡片显示新头像</t>
+          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,27 +1656,27 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>空名称预配置</t>
+          <t>回收孤儿任务</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
+          <t>处理中卡片点「编辑」→ 状态改为「待处理」→ 保存（或 `curl -X POST http://localhost:8080/api/tasks/&lt;id&gt;/recycle`）</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>名称自动等于 id</t>
+          <t>卡片回到**待处理**列，agent 头像消失</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>H4</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>预配置后，该 agent claim 时带别的名称/头像</t>
+          <t>回收后再点「接取」</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,7 +1730,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>回收</t>
+          <t>疑似卡住标记</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「回收」</t>
+          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,27 +1767,27 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,27 +1804,27 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,7 +1841,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>第一次 200，第二次 409 + error 信息</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,7 +1878,7 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
@@ -1888,17 +1888,17 @@
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>返回已归档任务数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,7 +1915,7 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,27 +1952,27 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>K. 跨平台（Mac）</t>
         </is>
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,27 +1989,27 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>K. 跨平台（Mac）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>Intel Mac</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,7 +2026,7 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>Gatekeeper</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>首次运行若提示"无法验证开发者"</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="0">
@@ -2063,7 +2063,7 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="0">
@@ -2073,17 +2073,17 @@
       </c>
       <c r="C55" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>系统选择</t>
         </is>
       </c>
       <c r="D55" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="0">
@@ -2092,80 +2092,6 @@
         </is>
       </c>
       <c r="G55" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr" s="0">
-        <is>
-          <t>K3</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr" s="0">
-        <is>
-          <t>K. 跨平台（Mac）</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr" s="0">
-        <is>
-          <t>Gatekeeper</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr" s="0">
-        <is>
-          <t>首次运行若提示"无法验证开发者"</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr" s="0">
-        <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr" s="0">
-        <is>
-          <t>K4</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr" s="0">
-        <is>
-          <t>K. 跨平台（Mac）</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr" s="0">
-        <is>
-          <t>系统选择</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr" s="0">
-        <is>
-          <t>Mac 上点「系统选择…」</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr" s="0">
-        <is>
-          <t>弹出 macOS 的 `choose folder` 对话框</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2173,7 +2099,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F57">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F55">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
ui: first-run onboarding wizard (same 4-step flow as README Quick Start); top-bar 使用向导 reopens it
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G58"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -250,27 +250,27 @@
     <row r="6">
       <c r="A6" t="inlineStr" s="0">
         <is>
-          <t>B1</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>A. 启动与页面</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t>正常添加</t>
+          <t>首次引导</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
         <is>
-          <t>点右上「＋ 添加任务」→ 弹窗填「任务标题」和「workspace 文件夹路径」→ 点「添加」</t>
+          <t>新开无痕窗口（或清掉 localStorage 里的 `lk-wizard-seen`）后打开页面</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，任务出现在**待处理**列（灰圈图标）</t>
+          <t>自动弹出「欢迎使用」引导向导，共 4 步，可「上一步 / 下一步 / 跳过」</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
@@ -287,27 +287,27 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="0">
         <is>
-          <t>B2</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>A. 启动与页面</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t>缺标题</t>
+          <t>重开向导</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>弹窗只填路径，点添加</t>
+          <t>向导里点「跳过」→ 点右上「使用向导」</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t>弹「添加任务失败：title is required」</t>
+          <t>向导关闭后，「使用向导」随时能重新打开</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
@@ -324,27 +324,27 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t>B3</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>A. 启动与页面</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t>缺路径</t>
+          <t>不再自动弹出</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>弹窗只填标题，点添加</t>
+          <t>点「跳过」或「开始使用」后刷新页面</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>弹「添加任务失败：workspacePath is required」</t>
+          <t>刷新后不再自动弹出（本浏览器记住；想要再看点「使用向导」）</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -361,7 +361,7 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>B4</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
@@ -371,17 +371,17 @@
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t>可选字段</t>
+          <t>正常添加</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t>添加时填描述、标签、截止时间</t>
+          <t>点右上「＋ 添加任务」→ 弹窗填「任务标题」和「workspace 文件夹路径」→ 点「添加」</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>卡片上显示紫色标签、黄色「截止…」提示、描述文本</t>
+          <t>弹窗关闭，任务出现在**待处理**列（灰圈图标）</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
@@ -398,7 +398,7 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t>B5</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
@@ -408,17 +408,17 @@
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t>多个标签</t>
+          <t>缺标题</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t>标签填 `go, ui`</t>
+          <t>弹窗只填路径，点添加</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>显示两个紫色标签</t>
+          <t>弹「添加任务失败：title is required」</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
@@ -435,7 +435,7 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="0">
         <is>
-          <t>B6</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
@@ -445,17 +445,17 @@
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t>截止时间留空</t>
+          <t>缺路径</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t>添加时不填截止时间</t>
+          <t>弹窗只填标题，点添加</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t>能正常添加，卡片无截止提示</t>
+          <t>弹「添加任务失败：workspacePath is required」</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
@@ -472,7 +472,7 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t>B7</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
@@ -482,17 +482,17 @@
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t>页内浏览选目录</t>
+          <t>可选字段</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="0">
         <is>
-          <t>点路径框旁「浏览…」→ 点进文件夹 → 点「选择此文件夹」</t>
+          <t>添加时填描述、标签、截止时间</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="0">
         <is>
-          <t>路径框自动填入所选文件夹的完整路径</t>
+          <t>卡片上显示紫色标签、黄色「截止…」提示、描述文本</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="0">
@@ -509,7 +509,7 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="0">
         <is>
-          <t>B8</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="0">
@@ -519,17 +519,17 @@
       </c>
       <c r="C13" t="inlineStr" s="0">
         <is>
-          <t>浏览上级</t>
+          <t>多个标签</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="0">
         <is>
-          <t>浏览弹窗里点「上级」</t>
+          <t>标签填 `go, ui`</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="0">
         <is>
-          <t>回到上一级目录；到根目录后显示 `C:\`、`D:\`（Mac 显示 `/`）</t>
+          <t>显示两个紫色标签</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="0">
@@ -546,7 +546,7 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="0">
         <is>
-          <t>B9</t>
+          <t>B6</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="0">
@@ -556,17 +556,17 @@
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t>系统选择</t>
+          <t>截止时间留空</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="0">
         <is>
-          <t>点「系统选择…」</t>
+          <t>添加时不填截止时间</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="0">
         <is>
-          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
+          <t>能正常添加，卡片无截止提示</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="0">
@@ -583,7 +583,7 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="0">
         <is>
-          <t>B10</t>
+          <t>B7</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="0">
@@ -593,17 +593,17 @@
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t>添加多个任务</t>
+          <t>页内浏览选目录</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
         <is>
-          <t>连续添加 2~3 个</t>
+          <t>点路径框旁「浏览…」→ 点进文件夹 → 点「选择此文件夹」</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="0">
         <is>
-          <t>都出现在待处理列，列标题右侧计数正确</t>
+          <t>路径框自动填入所选文件夹的完整路径</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="0">
@@ -620,7 +620,7 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="0">
         <is>
-          <t>B11</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="0">
@@ -630,17 +630,17 @@
       </c>
       <c r="C16" t="inlineStr" s="0">
         <is>
-          <t>直达项目目录</t>
+          <t>浏览上级</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="0">
         <is>
-          <t>点任意卡片标题旁的 📁 按钮</t>
+          <t>浏览弹窗里点「上级」</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="0">
         <is>
-          <t>服务器那台电脑弹出资源管理器/访达，定位到该任务的 workspace 文件夹；路径不存在时提示错误</t>
+          <t>回到上一级目录；到根目录后显示 `C:\`、`D:\`（Mac 显示 `/`）</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="0">
@@ -657,7 +657,7 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="0">
         <is>
-          <t>B12</t>
+          <t>B9</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
@@ -667,17 +667,17 @@
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t>取消添加</t>
+          <t>系统选择</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t>点「＋ 添加任务」→ 点「取消」或点弹窗外区域</t>
+          <t>点「系统选择…」</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，没有任务被创建</t>
+          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
@@ -694,27 +694,27 @@
     <row r="18">
       <c r="A18" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>B10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t>列标题图标</t>
+          <t>添加多个任务</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>看四个列标题前的圆圈</t>
+          <t>连续添加 2~3 个</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
+          <t>都出现在待处理列，列标题右侧计数正确</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
@@ -731,27 +731,27 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>无整条色带</t>
+          <t>直达项目目录</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t>看列头背景</t>
+          <t>点任意卡片标题旁的 📁 按钮</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>列头是白底细边，不是一整条颜色</t>
+          <t>服务器那台电脑弹出资源管理器/访达，定位到该任务的 workspace 文件夹；路径不存在时提示错误</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
@@ -768,27 +768,27 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>主界面无注册入口</t>
+          <t>取消添加</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>点「＋ 添加任务」→ 点「取消」或点弹窗外区域</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>页面上**没有**「Agent 管理 / 注册」表单；agent 信息只出现在被它接取的卡片上</t>
+          <t>弹窗关闭，没有任务被创建</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,27 +805,27 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 四列看板</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>API 注册并接取</t>
+          <t>列标题图标</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>先上传头像：`curl -F "file=@头像.png" http://localhost:8080/api/avatars`，记下返回的 `path`；再 claim：`curl -X POST -H "Content-Type: application/json" -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;上一步的path&gt;"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`</t>
+          <t>看四个列标题前的圆圈</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>返回 200，卡片移到**处理中**列，标题旁显示图片头像 + 名称</t>
+          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,27 +842,27 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 四列看板</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>卡片只显示名称</t>
+          <t>无整条色带</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>用名称 `Grok Build`、id `grok build` 接取后看卡片</t>
+          <t>看列头背景</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>卡片只显示图片头像 + 加粗名称「Grok Build」，**不显示** id（id 仅存在于 API 层）</t>
+          <t>列头是白底细边，不是一整条颜色</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,7 +879,7 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
@@ -889,17 +889,17 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>图片头像</t>
+          <t>主界面无注册入口</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>接取后看卡片</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>显示上传的图片（圆形裁剪），不是字母/表情符号</t>
+          <t>页面上**没有**「Agent 管理 / 注册」表单；agent 信息只出现在被它接取的卡片上</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,7 +916,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
@@ -926,17 +926,17 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>缺名称/头像被拒</t>
+          <t>API 注册并接取</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
+          <t>先上传头像：`curl -F "file=@头像.png" http://localhost:8080/api/avatars`，记下返回的 `path`；再 claim：`curl -X POST -H "Content-Type: application/json" -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;上一步的path&gt;"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
+          <t>返回 200，卡片移到**处理中**列，标题旁显示图片头像 + 名称</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,7 +953,7 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
@@ -963,17 +963,17 @@
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>多个 agent</t>
+          <t>卡片只显示名称</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>换一个 agentId 接取另一个任务</t>
+          <t>用名称 `Grok Build`、id `grok build` 接取后看卡片</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>每个卡片显示各自的 agent 头像</t>
+          <t>卡片只显示图片头像 + 加粗名称「Grok Build」，**不显示** id（id 仅存在于 API 层）</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,7 +990,7 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
@@ -1000,17 +1000,17 @@
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>图片头像</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>两个不同 agentId 先后 claim 同一任务（或开两个浏览器窗口同时点）</t>
+          <t>接取后看卡片</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>**只有一个人成功**，另一个 409 + 提示</t>
+          <t>显示上传的图片（圆形裁剪），不是字母/表情符号</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,27 +1027,27 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
         <is>
-          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>处理中/阻碍卡片按钮</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>看「处理中」「遇到阻碍」列的卡片</t>
+          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>只显示「编辑」「删除」，没有「阻碍/完成/回收/解除阻碍」按钮</t>
+          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,27 +1064,27 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
         <is>
-          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>API 状态流转</t>
+          <t>多个 agent</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>用 curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
+          <t>换一个 agentId 接取另一个任务</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>卡片在列间正确移动（这是 agent 的动作，界面不提供按钮）</t>
+          <t>每个卡片显示各自的 agent 头像</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,27 +1101,27 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>等你确认的卡片点「验收通过（归档）」</t>
+          <t>两个不同 agentId 先后 claim 同一任务（或开两个浏览器窗口同时点）</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
+          <t>**只有一个人成功**，另一个 409 + 提示</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,27 +1138,27 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>无退回修改按钮</t>
+          <t>处理中/阻碍卡片按钮</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>看「等你确认」卡片</t>
+          <t>看「处理中」「遇到阻碍」列的卡片</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>只有「验收通过（归档）」「编辑」「删除」，没有「退回修改」——要退回时直接命令 agent，agent 自己调 API 把任务退回「处理中」</t>
+          <t>只显示「编辑」「删除」，没有「阻碍/完成/回收/解除阻碍」按钮</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,27 +1175,27 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>API 状态流转</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>归档历史弹窗里看条目</t>
+          <t>用 curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>显示标题、标签、完成时间</t>
+          <t>卡片在列间正确移动（这是 agent 的动作，界面不提供按钮）</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,7 +1212,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>历史关闭</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>点「关闭」或点击弹窗外区域</t>
+          <t>等你确认的卡片点「验收通过（归档）」</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，看板恢复正常</t>
+          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,7 +1249,7 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>F5</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
@@ -1259,17 +1259,17 @@
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>单条删除</t>
+          <t>无退回修改按钮</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗里点某条「删除」→ 确认</t>
+          <t>看「等你确认」卡片</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>该条消失，看板和历史里都不再有</t>
+          <t>只有「验收通过（归档）」「编辑」「删除」，没有「退回修改」——要退回时直接命令 agent，agent 自己调 API 把任务退回「处理中」</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,7 +1286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>F6</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1296,17 +1296,17 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>全选删除</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
+          <t>归档历史弹窗里看条目</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>选中的条目全部消失</t>
+          <t>显示标题、标签、完成时间</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,27 +1323,27 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>编辑字段</t>
+          <t>历史关闭</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
+          <t>点「关闭」或点击弹窗外区域</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>卡片内容更新</t>
+          <t>弹窗关闭，看板恢复正常</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,27 +1360,27 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
+          <t>历史弹窗里点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>该条消失，看板和历史里都不再有</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,27 +1397,27 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>全选删除</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>编辑里把标签清空 → 保存</t>
+          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>卡片上的标签消失</t>
+          <t>选中的条目全部消失</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,7 +1434,7 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>编辑字段</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「删除」→ 确认弹窗</t>
+          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
+          <t>卡片内容更新</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,7 +1471,7 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>G5</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>编辑已归档任务</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>历史里没有编辑入口</t>
+          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>归档历史只读（符合预期）</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,27 +1508,27 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
+          <t>编辑里把标签清空 → 保存</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
+          <t>卡片上的标签消失</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
+          <t>任意卡片点「删除」→ 确认弹窗</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>之后该 agent 接取的卡片显示新头像</t>
+          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,27 +1582,27 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>空名称预配置</t>
+          <t>编辑已归档任务</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
+          <t>历史里没有编辑入口</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>名称自动等于 id</t>
+          <t>归档历史只读（符合预期）</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,7 +1619,7 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>H4</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
@@ -1629,17 +1629,17 @@
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>预配置后，该 agent claim 时带别的名称/头像</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
+          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,27 +1656,27 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>回收孤儿任务</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「编辑」→ 状态改为「待处理」→ 保存（或 `curl -X POST http://localhost:8080/api/tasks/&lt;id&gt;/recycle`）</t>
+          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>之后该 agent 接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>空名称预配置</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>名称自动等于 id</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,27 +1730,27 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>预配置后，该 agent claim 时带别的名称/头像</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,27 +1767,27 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>回收孤儿任务</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>处理中卡片点「编辑」→ 状态改为「待处理」→ 保存（或 `curl -X POST http://localhost:8080/api/tasks/&lt;id&gt;/recycle`）</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>卡片回到**待处理**列，agent 头像消失</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,27 +1804,27 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>回收后再点「接取」</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,27 +1841,27 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>疑似卡住标记</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,7 +1878,7 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
@@ -1888,17 +1888,17 @@
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,7 +1915,7 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,27 +1952,27 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>第一次 200，第二次 409 + error 信息</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,27 +1989,27 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>返回已归档任务数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,27 +2026,27 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t>Gatekeeper</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
         <is>
-          <t>首次运行若提示"无法验证开发者"</t>
+          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="0">
         <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="0">
@@ -2063,35 +2063,146 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="0">
+        <is>
+          <t>Apple Silicon</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="0">
+        <is>
+          <t>正常启动，页面功能同 Windows</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr" s="0">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr" s="0">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr" s="0">
+        <is>
+          <t>Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr" s="0">
+        <is>
+          <t>首次运行若提示"无法验证开发者"</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr" s="0">
+        <is>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr" s="0">
+        <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr" s="0">
+      <c r="B58" t="inlineStr" s="0">
         <is>
           <t>K. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr" s="0">
+      <c r="C58" t="inlineStr" s="0">
         <is>
           <t>系统选择</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr" s="0">
+      <c r="D58" t="inlineStr" s="0">
         <is>
           <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr" s="0">
+      <c r="E58" t="inlineStr" s="0">
         <is>
           <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr" s="0">
+      <c r="F58" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2099,7 +2210,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F55">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F58">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: bilingual UI (zh/en with top-bar toggle, browser auto-detect); README split into English + 中文 (README_CN) with cross-links and downloads; About metadata; checklist xlsx generator accepts suffixed row ids (A1b/A6b)
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G60"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -139,7 +139,7 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="0">
         <is>
-          <t>A2</t>
+          <t>A1b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="0">
@@ -149,17 +149,17 @@
       </c>
       <c r="C3" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>双击启动</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="0">
         <is>
-          <t>浏览器开 http://localhost:8080/api/health</t>
+          <t>直接双击 `dist\light-kanban.exe`</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>显示 `{"db":"ok","status":"ok"}`</t>
+          <t>弹出控制台窗口并**自动打开浏览器** http://localhost:8080，控制台打印访问地址</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
@@ -176,7 +176,7 @@
     <row r="4">
       <c r="A4" t="inlineStr" s="0">
         <is>
-          <t>A3</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="0">
@@ -186,17 +186,17 @@
       </c>
       <c r="C4" t="inlineStr" s="0">
         <is>
-          <t>页面加载</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="0">
         <is>
-          <t>打开 http://localhost:8080</t>
+          <t>浏览器开 http://localhost:8080/api/health</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>出现「Light-Kanban 任务看板」标题，**没有**弹窗盖住页面</t>
+          <t>显示 `{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="0">
@@ -213,7 +213,7 @@
     <row r="5">
       <c r="A5" t="inlineStr" s="0">
         <is>
-          <t>A4</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="0">
@@ -223,17 +223,17 @@
       </c>
       <c r="C5" t="inlineStr" s="0">
         <is>
-          <t>连接指示</t>
+          <t>页面加载</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="0">
         <is>
-          <t>看右上角圆点</t>
+          <t>打开 http://localhost:8080</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t>绿色 ●</t>
+          <t>出现「Light-Kanban 任务看板」标题，**没有**弹窗盖住页面</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="0">
@@ -250,7 +250,7 @@
     <row r="6">
       <c r="A6" t="inlineStr" s="0">
         <is>
-          <t>A5</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="0">
@@ -260,17 +260,17 @@
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t>首次引导</t>
+          <t>连接指示</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
         <is>
-          <t>新开无痕窗口（或清掉 localStorage 里的 `lk-wizard-seen`）后打开页面</t>
+          <t>看右上角圆点</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>自动弹出「欢迎使用」引导向导，共 4 步，可「上一步 / 下一步 / 跳过」</t>
+          <t>绿色 ●</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
@@ -287,7 +287,7 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="0">
         <is>
-          <t>A6</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
@@ -297,17 +297,17 @@
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t>重开向导</t>
+          <t>首次引导</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>向导里点「跳过」→ 点右上「使用向导」</t>
+          <t>新开无痕窗口（或清掉 localStorage 里的 `lk-wizard-seen`）后打开页面</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t>向导关闭后，「使用向导」随时能重新打开</t>
+          <t>自动弹出「欢迎使用」引导向导，共 4 步，可「上一步 / 下一步 / 跳过」</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
@@ -324,7 +324,7 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t>A7</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
@@ -334,17 +334,17 @@
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t>不再自动弹出</t>
+          <t>重开向导</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>点「跳过」或「开始使用」后刷新页面</t>
+          <t>向导里点「跳过」→ 点右上「使用向导」</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>刷新后不再自动弹出（本浏览器记住；想要再看点「使用向导」）</t>
+          <t>向导关闭后，「使用向导」随时能重新打开</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -361,27 +361,27 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>B1</t>
+          <t>A6b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>A. 启动与页面</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t>正常添加</t>
+          <t>语言切换</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t>点右上「＋ 添加任务」→ 弹窗填「任务标题」和「workspace 文件夹路径」→ 点「添加」</t>
+          <t>点顶栏「EN / 中文」按钮</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，任务出现在**待处理**列（灰圈图标）</t>
+          <t>整个界面（列名、按钮、弹窗、向导）在中英文间即时切换；刷新后保持所选语言</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
@@ -398,27 +398,27 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t>B2</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>A. 启动与页面</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t>缺标题</t>
+          <t>不再自动弹出</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t>弹窗只填路径，点添加</t>
+          <t>点「跳过」或「开始使用」后刷新页面</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>弹「添加任务失败：title is required」</t>
+          <t>刷新后不再自动弹出（本浏览器记住；想要再看点「使用向导」）</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
@@ -435,7 +435,7 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="0">
         <is>
-          <t>B3</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
@@ -445,17 +445,17 @@
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t>缺路径</t>
+          <t>正常添加</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t>弹窗只填标题，点添加</t>
+          <t>点右上「＋ 添加任务」→ 弹窗填「任务标题」和「workspace 文件夹路径」→ 点「添加」</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t>弹「添加任务失败：workspacePath is required」</t>
+          <t>弹窗关闭，任务出现在**待处理**列（灰圈图标）</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
@@ -472,7 +472,7 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t>B4</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
@@ -482,17 +482,17 @@
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t>可选字段</t>
+          <t>缺标题</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="0">
         <is>
-          <t>添加时填描述、标签、截止时间</t>
+          <t>弹窗只填路径，点添加</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="0">
         <is>
-          <t>卡片上显示紫色标签、黄色「截止…」提示、描述文本</t>
+          <t>弹「添加任务失败：title is required」</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="0">
@@ -509,7 +509,7 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="0">
         <is>
-          <t>B5</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="0">
@@ -519,17 +519,17 @@
       </c>
       <c r="C13" t="inlineStr" s="0">
         <is>
-          <t>多个标签</t>
+          <t>缺路径</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="0">
         <is>
-          <t>标签填 `go, ui`</t>
+          <t>弹窗只填标题，点添加</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="0">
         <is>
-          <t>显示两个紫色标签</t>
+          <t>弹「添加任务失败：workspacePath is required」</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="0">
@@ -546,7 +546,7 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="0">
         <is>
-          <t>B6</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="0">
@@ -556,17 +556,17 @@
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t>截止时间留空</t>
+          <t>可选字段</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="0">
         <is>
-          <t>添加时不填截止时间</t>
+          <t>添加时填描述、标签、截止时间</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="0">
         <is>
-          <t>能正常添加，卡片无截止提示</t>
+          <t>卡片上显示紫色标签、黄色「截止…」提示、描述文本</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="0">
@@ -583,7 +583,7 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="0">
         <is>
-          <t>B7</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="0">
@@ -593,17 +593,17 @@
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t>页内浏览选目录</t>
+          <t>多个标签</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
         <is>
-          <t>点路径框旁「浏览…」→ 点进文件夹 → 点「选择此文件夹」</t>
+          <t>标签填 `go, ui`</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="0">
         <is>
-          <t>路径框自动填入所选文件夹的完整路径</t>
+          <t>显示两个紫色标签</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="0">
@@ -620,7 +620,7 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="0">
         <is>
-          <t>B8</t>
+          <t>B6</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="0">
@@ -630,17 +630,17 @@
       </c>
       <c r="C16" t="inlineStr" s="0">
         <is>
-          <t>浏览上级</t>
+          <t>截止时间留空</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="0">
         <is>
-          <t>浏览弹窗里点「上级」</t>
+          <t>添加时不填截止时间</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="0">
         <is>
-          <t>回到上一级目录；到根目录后显示 `C:\`、`D:\`（Mac 显示 `/`）</t>
+          <t>能正常添加，卡片无截止提示</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="0">
@@ -657,7 +657,7 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="0">
         <is>
-          <t>B9</t>
+          <t>B7</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
@@ -667,17 +667,17 @@
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t>系统选择</t>
+          <t>页内浏览选目录</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t>点「系统选择…」</t>
+          <t>点路径框旁「浏览…」→ 点进文件夹 → 点「选择此文件夹」</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
+          <t>路径框自动填入所选文件夹的完整路径</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
@@ -694,7 +694,7 @@
     <row r="18">
       <c r="A18" t="inlineStr" s="0">
         <is>
-          <t>B10</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
@@ -704,17 +704,17 @@
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t>添加多个任务</t>
+          <t>浏览上级</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>连续添加 2~3 个</t>
+          <t>浏览弹窗里点「上级」</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>都出现在待处理列，列标题右侧计数正确</t>
+          <t>回到上一级目录；到根目录后显示 `C:\`、`D:\`（Mac 显示 `/`）</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
@@ -731,7 +731,7 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="0">
         <is>
-          <t>B11</t>
+          <t>B9</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
@@ -741,17 +741,17 @@
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>直达项目目录</t>
+          <t>系统选择</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t>点任意卡片标题旁的 📁 按钮</t>
+          <t>点「系统选择…」</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>服务器那台电脑弹出资源管理器/访达，定位到该任务的 workspace 文件夹；路径不存在时提示错误</t>
+          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
@@ -768,7 +768,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>B12</t>
+          <t>B10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
@@ -778,17 +778,17 @@
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>取消添加</t>
+          <t>添加多个任务</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>点「＋ 添加任务」→ 点「取消」或点弹窗外区域</t>
+          <t>连续添加 2~3 个</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，没有任务被创建</t>
+          <t>都出现在待处理列，列标题右侧计数正确</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,27 +805,27 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>列标题图标</t>
+          <t>直达项目目录</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>看四个列标题前的圆圈</t>
+          <t>点任意卡片标题旁的 📁 按钮</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
+          <t>服务器那台电脑弹出资源管理器/访达，定位到该任务的 workspace 文件夹；路径不存在时提示错误</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,27 +842,27 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>B. 添加任务</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>无整条色带</t>
+          <t>取消添加</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>看列头背景</t>
+          <t>点「＋ 添加任务」→ 点「取消」或点弹窗外区域</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>列头是白底细边，不是一整条颜色</t>
+          <t>弹窗关闭，没有任务被创建</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,27 +879,27 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 四列看板</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>主界面无注册入口</t>
+          <t>列标题图标</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>看四个列标题前的圆圈</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>页面上**没有**「Agent 管理 / 注册」表单；agent 信息只出现在被它接取的卡片上</t>
+          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,27 +916,27 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 四列看板</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>API 注册并接取</t>
+          <t>无整条色带</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>先上传头像：`curl -F "file=@头像.png" http://localhost:8080/api/avatars`，记下返回的 `path`；再 claim：`curl -X POST -H "Content-Type: application/json" -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;上一步的path&gt;"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`</t>
+          <t>看列头背景</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>返回 200，卡片移到**处理中**列，标题旁显示图片头像 + 名称</t>
+          <t>列头是白底细边，不是一整条颜色</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,7 +953,7 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
@@ -963,17 +963,17 @@
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>卡片只显示名称</t>
+          <t>主界面无注册入口</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>用名称 `Grok Build`、id `grok build` 接取后看卡片</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>卡片只显示图片头像 + 加粗名称「Grok Build」，**不显示** id（id 仅存在于 API 层）</t>
+          <t>页面上**没有**「Agent 管理 / 注册」表单；agent 信息只出现在被它接取的卡片上</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,7 +990,7 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
@@ -1000,17 +1000,17 @@
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>图片头像</t>
+          <t>API 注册并接取</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>接取后看卡片</t>
+          <t>先上传头像：`curl -F "file=@头像.png" http://localhost:8080/api/avatars`，记下返回的 `path`；再 claim：`curl -X POST -H "Content-Type: application/json" -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;上一步的path&gt;"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>显示上传的图片（圆形裁剪），不是字母/表情符号</t>
+          <t>返回 200，卡片移到**处理中**列，标题旁显示图片头像 + 名称</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,7 +1027,7 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>缺名称/头像被拒</t>
+          <t>卡片只显示名称</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
+          <t>用名称 `Grok Build`、id `grok build` 接取后看卡片</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
+          <t>卡片只显示图片头像 + 加粗名称「Grok Build」，**不显示** id（id 仅存在于 API 层）</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,7 +1064,7 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>多个 agent</t>
+          <t>图片头像</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>换一个 agentId 接取另一个任务</t>
+          <t>接取后看卡片</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>每个卡片显示各自的 agent 头像</t>
+          <t>显示上传的图片（圆形裁剪），不是字母/表情符号</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,7 +1101,7 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>两个不同 agentId 先后 claim 同一任务（或开两个浏览器窗口同时点）</t>
+          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>**只有一个人成功**，另一个 409 + 提示</t>
+          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,27 +1138,27 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>处理中/阻碍卡片按钮</t>
+          <t>多个 agent</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>看「处理中」「遇到阻碍」列的卡片</t>
+          <t>换一个 agentId 接取另一个任务</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>只显示「编辑」「删除」，没有「阻碍/完成/回收/解除阻碍」按钮</t>
+          <t>每个卡片显示各自的 agent 头像</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,27 +1175,27 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
         <is>
-          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
+          <t>D. 接取任务 &amp; agent 身份</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>API 状态流转</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>用 curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
+          <t>两个不同 agentId 先后 claim 同一任务（或开两个浏览器窗口同时点）</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>卡片在列间正确移动（这是 agent 的动作，界面不提供按钮）</t>
+          <t>**只有一个人成功**，另一个 409 + 提示</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,27 +1212,27 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>处理中/阻碍卡片按钮</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>等你确认的卡片点「验收通过（归档）」</t>
+          <t>看「处理中」「遇到阻碍」列的卡片</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
+          <t>只显示「编辑」「删除」，没有「阻碍/完成/回收/解除阻碍」按钮</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,27 +1249,27 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>无退回修改按钮</t>
+          <t>API 状态流转</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>看「等你确认」卡片</t>
+          <t>用 curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>只有「验收通过（归档）」「编辑」「删除」，没有「退回修改」——要退回时直接命令 agent，agent 自己调 API 把任务退回「处理中」</t>
+          <t>卡片在列间正确移动（这是 agent 的动作，界面不提供按钮）</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,7 +1286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1296,17 +1296,17 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>归档历史弹窗里看条目</t>
+          <t>等你确认的卡片点「验收通过（归档）」</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>显示标题、标签、完成时间</t>
+          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,7 +1323,7 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
@@ -1333,17 +1333,17 @@
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>历史关闭</t>
+          <t>无退回修改按钮</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>点「关闭」或点击弹窗外区域</t>
+          <t>看「等你确认」卡片</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，看板恢复正常</t>
+          <t>只有「验收通过（归档）」「编辑」「删除」，没有「退回修改」——要退回时直接命令 agent，agent 自己调 API 把任务退回「处理中」</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,7 +1360,7 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>F5</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
@@ -1370,17 +1370,17 @@
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>单条删除</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗里点某条「删除」→ 确认</t>
+          <t>归档历史弹窗里看条目</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>该条消失，看板和历史里都不再有</t>
+          <t>显示标题、标签、完成时间</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,7 +1397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>F6</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>全选删除</t>
+          <t>历史关闭</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
+          <t>点「关闭」或点击弹窗外区域</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>选中的条目全部消失</t>
+          <t>弹窗关闭，看板恢复正常</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,27 +1434,27 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>编辑字段</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
+          <t>历史弹窗里点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>卡片内容更新</t>
+          <t>该条消失，看板和历史里都不再有</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,27 +1471,27 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>全选删除</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
+          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>选中的条目全部消失</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,7 +1508,7 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>编辑字段</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>编辑里把标签清空 → 保存</t>
+          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>卡片上的标签消失</t>
+          <t>卡片内容更新</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,7 +1545,7 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
@@ -1555,17 +1555,17 @@
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「删除」→ 确认弹窗</t>
+          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,7 +1582,7 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>G5</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>编辑已归档任务</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>历史里没有编辑入口</t>
+          <t>编辑里把标签清空 → 保存</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>归档历史只读（符合预期）</t>
+          <t>卡片上的标签消失</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,27 +1619,27 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
+          <t>任意卡片点「删除」→ 确认弹窗</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
+          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,27 +1656,27 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 编辑任务</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>编辑已归档任务</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
+          <t>历史里没有编辑入口</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>之后该 agent 接取的卡片显示新头像</t>
+          <t>归档历史只读（符合预期）</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,7 +1693,7 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
@@ -1703,17 +1703,17 @@
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>空名称预配置</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>名称自动等于 id</t>
+          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,7 +1730,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>H4</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>预配置后，该 agent claim 时带别的名称/头像</t>
+          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
+          <t>之后该 agent 接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,27 +1767,27 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>回收孤儿任务</t>
+          <t>空名称预配置</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「编辑」→ 状态改为「待处理」→ 保存（或 `curl -X POST http://localhost:8080/api/tasks/&lt;id&gt;/recycle`）</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>名称自动等于 id</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,27 +1804,27 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. Agent 身份（API 预配置）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>预配置后，该 agent claim 时带别的名称/头像</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,7 +1841,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>回收孤儿任务</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>处理中卡片点「编辑」→ 状态改为「待处理」→ 保存（或 `curl -X POST http://localhost:8080/api/tasks/&lt;id&gt;/recycle`）</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>卡片回到**待处理**列，agent 头像消失</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,27 +1878,27 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>回收后再点「接取」</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,27 +1915,27 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>疑似卡住标记</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,7 +1952,7 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,7 +1989,7 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
@@ -1999,17 +1999,17 @@
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,7 +2026,7 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>第一次 200，第二次 409 + error 信息</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="0">
@@ -2063,27 +2063,27 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C55" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D55" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>返回已归档任务数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="0">
@@ -2100,27 +2100,27 @@
     <row r="56">
       <c r="A56" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C56" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D56" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
         </is>
       </c>
       <c r="E56" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="0">
@@ -2137,7 +2137,7 @@
     <row r="57">
       <c r="A57" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="0">
@@ -2147,17 +2147,17 @@
       </c>
       <c r="C57" t="inlineStr" s="0">
         <is>
-          <t>Gatekeeper</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="0">
         <is>
-          <t>首次运行若提示"无法验证开发者"</t>
+          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="0">
         <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="0">
@@ -2174,35 +2174,109 @@
     <row r="58">
       <c r="A58" t="inlineStr" s="0">
         <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr" s="0">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr" s="0">
+        <is>
+          <t>K. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr" s="0">
+        <is>
+          <t>Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr" s="0">
+        <is>
+          <t>首次运行若提示"无法验证开发者"</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr" s="0">
+        <is>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr" s="0">
+        <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr" s="0">
+      <c r="B60" t="inlineStr" s="0">
         <is>
           <t>K. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr" s="0">
+      <c r="C60" t="inlineStr" s="0">
         <is>
           <t>系统选择</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr" s="0">
+      <c r="D60" t="inlineStr" s="0">
         <is>
           <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr" s="0">
+      <c r="E60" t="inlineStr" s="0">
         <is>
           <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr" s="0">
+      <c r="F60" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2210,7 +2284,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F58">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F60">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: sync all documentation with the v1.0.2 React UI
README/README_CN: new UI walkthrough (topbar, drawer review flow, search
& filters), React dev commands, block reason / reject feedback examples.
AGENTS: new layout, frontend toolchain, conventions. CONTEXT: task
drawer, request changes, block reason, workspace filter, short id.
spec.md: blockReason/reviewFeedback schema + API rows, Web UI paragraph,
recycle paths. checklist: rewritten for the new UI (76 rows) and xlsx
regenerated. ADR-0002: React frontend decision. cross-build.ps1: build
and stage the frontend before compiling.
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G77"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -117,7 +117,7 @@
       </c>
       <c r="D2" t="inlineStr" s="0">
         <is>
-          <t>运行 `dist\light-kanban.exe -addr :8080`</t>
+          <t>运行 `./dist/light-kanban -addr :8080`</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="0">
@@ -149,7 +149,7 @@
       </c>
       <c r="C3" t="inlineStr" s="0">
         <is>
-          <t>双击启动</t>
+          <t>双击启动（Windows）</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="0">
@@ -159,7 +159,7 @@
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>弹出控制台窗口并**自动打开浏览器** http://localhost:8080，控制台打印访问地址</t>
+          <t>弹出控制台窗口并**自动打开浏览器** http://localhost:8080</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
@@ -233,7 +233,7 @@
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t>出现「Light-Kanban 任务看板」标题，**没有**弹窗盖住页面</t>
+          <t>浅色顶栏（Light Kanban / 任务看板）+ 四列看板，无弹窗遮盖，无深色大 Header</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="0">
@@ -265,12 +265,12 @@
       </c>
       <c r="D6" t="inlineStr" s="0">
         <is>
-          <t>看右上角圆点</t>
+          <t>正常时看顶栏右侧</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>绿色 ●</t>
+          <t>**没有**常亮绿色状态点；停掉服务后出现红色「连接失败」</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
@@ -302,12 +302,12 @@
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>新开无痕窗口（或清掉 localStorage 里的 `lk-wizard-seen`）后打开页面</t>
+          <t>新开无痕窗口（或清掉 localStorage `lk-wizard-seen`）打开页面</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t>自动弹出「欢迎使用」引导向导，共 4 步，可「上一步 / 下一步 / 跳过」</t>
+          <t>自动弹出 4 步引导向导，可上一步 / 下一步 / 跳过</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
@@ -339,12 +339,12 @@
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>向导里点「跳过」→ 点右上「使用向导」</t>
+          <t>跳过向导 → 顶栏右侧设置（齿轮）→「使用向导」</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>向导关闭后，「使用向导」随时能重新打开</t>
+          <t>向导随时能重新打开</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -376,12 +376,12 @@
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t>点顶栏「EN / 中文」按钮</t>
+          <t>设置菜单 →「界面语言」</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>整个界面（列名、按钮、弹窗、向导）在中英文间即时切换；刷新后保持所选语言</t>
+          <t>整个界面（列名、按钮、弹窗、抽屉、向导）在中英文间即时切换；刷新后保持</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
@@ -418,7 +418,7 @@
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>刷新后不再自动弹出（本浏览器记住；想要再看点「使用向导」）</t>
+          <t>刷新后不再自动弹出</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
@@ -440,22 +440,22 @@
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t>正常添加</t>
+          <t>顶栏新建</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t>点右上「＋ 添加任务」→ 弹窗填「任务标题」和「workspace 文件夹路径」→ 点「添加」</t>
+          <t>点顶栏右侧「+」→ 填标题和 workspace 路径 → 创建</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，任务出现在**待处理**列（灰圈图标）</t>
+          <t>弹窗关闭，任务出现在**待处理**列</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
@@ -472,27 +472,27 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t>B2</t>
+          <t>B1b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t>缺标题</t>
+          <t>列头快速新增</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="0">
         <is>
-          <t>弹窗只填路径，点添加</t>
+          <t>点待处理列标题右侧「+」</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="0">
         <is>
-          <t>弹「添加任务失败：title is required」</t>
+          <t>同样打开新建弹窗，创建后进入待处理列</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="0">
@@ -509,27 +509,27 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="0">
         <is>
-          <t>B3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="0">
         <is>
-          <t>缺路径</t>
+          <t>缺标题</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="0">
         <is>
-          <t>弹窗只填标题，点添加</t>
+          <t>弹窗只填路径，点创建</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="0">
         <is>
-          <t>弹「添加任务失败：workspacePath is required」</t>
+          <t>弹「创建任务失败：title is required」</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="0">
@@ -546,27 +546,27 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="0">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t>可选字段</t>
+          <t>缺路径</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="0">
         <is>
-          <t>添加时填描述、标签、截止时间</t>
+          <t>弹窗只填标题，点创建</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="0">
         <is>
-          <t>卡片上显示紫色标签、黄色「截止…」提示、描述文本</t>
+          <t>弹「创建任务失败：workspacePath is required」</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="0">
@@ -583,27 +583,27 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="0">
         <is>
-          <t>B5</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t>多个标签</t>
+          <t>可选字段</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
         <is>
-          <t>标签填 `go, ui`</t>
+          <t>填描述、标签、截止时间</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="0">
         <is>
-          <t>显示两个紫色标签</t>
+          <t>卡片显示标签、截止提示；描述在抽屉里完整可见</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="0">
@@ -620,27 +620,27 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="0">
         <is>
-          <t>B6</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="0">
         <is>
-          <t>截止时间留空</t>
+          <t>多个标签</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="0">
         <is>
-          <t>添加时不填截止时间</t>
+          <t>标签填 `go, ui, test`</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="0">
         <is>
-          <t>能正常添加，卡片无截止提示</t>
+          <t>卡片最多显示 2 个标签 + 「+1」</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="0">
@@ -657,27 +657,27 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="0">
         <is>
-          <t>B7</t>
+          <t>B6</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t>页内浏览选目录</t>
+          <t>截止时间留空</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t>点路径框旁「浏览…」→ 点进文件夹 → 点「选择此文件夹」</t>
+          <t>不填截止时间</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>路径框自动填入所选文件夹的完整路径</t>
+          <t>能正常创建，卡片无截止提示</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
@@ -694,27 +694,27 @@
     <row r="18">
       <c r="A18" t="inlineStr" s="0">
         <is>
-          <t>B8</t>
+          <t>B7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t>浏览上级</t>
+          <t>页内浏览选目录</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>浏览弹窗里点「上级」</t>
+          <t>点路径框旁「浏览…」→ 点进文件夹 →「选择此文件夹」</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>回到上一级目录；到根目录后显示 `C:\`、`D:\`（Mac 显示 `/`）</t>
+          <t>路径框自动填入所选文件夹完整路径</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
@@ -731,27 +731,27 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="0">
         <is>
-          <t>B9</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>系统选择</t>
+          <t>浏览上级</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t>点「系统选择…」</t>
+          <t>浏览弹窗里点「上级」</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
+          <t>回到上一级目录；到根目录后 Mac 显示 `/`</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
@@ -768,27 +768,27 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>B10</t>
+          <t>B9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>添加多个任务</t>
+          <t>系统选择</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>连续添加 2~3 个</t>
+          <t>点「系统选择…」</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>都出现在待处理列，列标题右侧计数正确</t>
+          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,27 +805,27 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>B11</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>直达项目目录</t>
+          <t>取消新建</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>点任意卡片标题旁的 📁 按钮</t>
+          <t>打开弹窗后点「取消」/ 点弹窗外 / 按 Esc</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>服务器那台电脑弹出资源管理器/访达，定位到该任务的 workspace 文件夹；路径不存在时提示错误</t>
+          <t>弹窗关闭，没有任务被创建</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,27 +842,27 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>B12</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
         <is>
-          <t>B. 添加任务</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>取消添加</t>
+          <t>四列结构</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>点「＋ 添加任务」→ 点「取消」或点弹窗外区域</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，没有任务被创建</t>
+          <t>待处理(灰○) / 处理中(黄◐) / 遇到阻碍(红!) / 等你确认(绿✓)，列头右侧有任务计数</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,27 +879,27 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>列标题图标</t>
+          <t>列独立滚动</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>看四个列标题前的圆圈</t>
+          <t>灌入演示数据后滚动某一列</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>待处理=灰色空心圆，处理中=黄色圆(…)，遇到阻碍=红色圆(!)，等你确认=绿色圆(✓)</t>
+          <t>每列独立上下滚动，页面整体不随任务增多向下增长</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,27 +916,27 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
         <is>
-          <t>C. 四列看板</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>无整条色带</t>
+          <t>列头固定</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>看列头背景</t>
+          <t>列内滚动时看列头</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>列头是白底细边，不是一整条颜色</t>
+          <t>列标题、计数、快速新增按钮始终停在列顶</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,27 +953,27 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>主界面无注册入口</t>
+          <t>窄屏横滚</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>把窗口拖窄（&lt; ~1300px）</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>页面上**没有**「Agent 管理 / 注册」表单；agent 信息只出现在被它接取的卡片上</t>
+          <t>看板出现横向滚动，四列保持原宽度不重排</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,27 +990,27 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>API 注册并接取</t>
+          <t>高密度</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>先上传头像：`curl -F "file=@头像.png" http://localhost:8080/api/avatars`，记下返回的 `path`；再 claim：`curl -X POST -H "Content-Type: application/json" -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;上一步的path&gt;"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`</t>
+          <t>一屏内数卡片</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>返回 200，卡片移到**处理中**列，标题旁显示图片头像 + 名称</t>
+          <t>同样屏幕能放下明显比旧版更多的卡片，且不拥挤</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,27 +1027,27 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>卡片只显示名称</t>
+          <t>短号与头像</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>用名称 `Grok Build`、id `grok build` 接取后看卡片</t>
+          <t>看任意卡片第一行</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>卡片只显示图片头像 + 加粗名称「Grok Build」，**不显示** id（id 仅存在于 API 层）</t>
+          <t>左侧淡灰 `LK-XXXX` 短号，右侧 18px agent 头像（未接取的卡片没有头像）</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,27 +1064,27 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>图片头像</t>
+          <t>workspace 显示</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>接取后看卡片</t>
+          <t>看卡片底部</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>显示上传的图片（圆形裁剪），不是字母/表情符号</t>
+          <t>只显示文件夹名（如 light-kanban）+ 颜色点，**不显示**完整路径；悬停可见全路径</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,27 +1101,27 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>缺名称/头像被拒</t>
+          <t>标签折叠</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>API 接取时缺 `name`、头像不是图片（如 `G`、emoji）、或 `avatar` 指向不存在的文件（伪造 `/api/avatars/xxx.png`）</t>
+          <t>找一张 3+ 标签的卡</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>返回 422 并提示，任务不被接取，不会出现坏图</t>
+          <t>最多 2 个标签 + 「+N」，不撑高卡片</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,27 +1138,27 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>多个 agent</t>
+          <t>截止提示</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>换一个 agentId 接取另一个任务</t>
+          <t>演示数据里找今天截止 / 已逾期卡片</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>每个卡片显示各自的 agent 头像</t>
+          <t>分别显示黄色「今天截止」/ 红色「已逾期」；未来截止显示灰色短日期</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,27 +1175,27 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
         <is>
-          <t>D. 接取任务 &amp; agent 身份</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>卡住标记</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>两个不同 agentId 先后 claim 同一任务（或开两个浏览器窗口同时点）</t>
+          <t>处理中超过 24h 未更新的任务</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>**只有一个人成功**，另一个 409 + 提示</t>
+          <t>卡片底部出现「⚠ 疑似卡住」，无红框无闪烁</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,27 +1212,27 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
         <is>
-          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>处理中/阻碍卡片按钮</t>
+          <t>阻碍原因</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>看「处理中」「遇到阻碍」列的卡片</t>
+          <t>看遇到阻碍列卡片</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>只显示「编辑」「删除」，没有「阻碍/完成/回收/解除阻碍」按钮</t>
+          <t>卡片上直接以红色「! 原因」显示 agent 填的 blockReason</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,27 +1249,27 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
         <is>
-          <t>E. 状态流转（agent 通过 API 做，界面无按钮）</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>API 状态流转</t>
+          <t>长标题</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>用 curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
+          <t>找一张长标题卡</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>卡片在列间正确移动（这是 agent 的动作，界面不提供按钮）</t>
+          <t>标题最多两行截断，卡片不被撑爆</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,27 +1286,27 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>打开抽屉</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>等你确认的卡片点「验收通过（归档）」</t>
+          <t>点任意卡片</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；点右上「归档历史」→ 弹窗里能看到它，带「完成于 …」时间</t>
+          <t>右侧滑出抽屉，看板仍部分可见；含短号、标题、状态、Agent、workspace、描述、标签、截止、创建/更新时间</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,27 +1323,27 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>无退回修改按钮</t>
+          <t>关闭抽屉</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>看「等你确认」卡片</t>
+          <t>点 × / 点抽屉外 / 按 Esc</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>只有「验收通过（归档）」「编辑」「删除」，没有「退回修改」——要退回时直接命令 agent，agent 自己调 API 把任务退回「处理中」</t>
+          <t>抽屉关闭，回到原看板位置</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,27 +1360,27 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>查看/编辑分离</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>归档历史弹窗里看条目</t>
+          <t>打开抽屉</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>显示标题、标签、完成时间</t>
+          <t>默认是查看模式，没有输入框；点「编辑」才进入编辑</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,27 +1397,27 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>历史关闭</t>
+          <t>编辑保存</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>点「关闭」或点击弹窗外区域</t>
+          <t>编辑标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，看板恢复正常</t>
+          <t>回到查看模式，卡片内容更新</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,27 +1434,27 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>F5</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>单条删除</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗里点某条「删除」→ 确认</t>
+          <t>编辑里把状态从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>该条消失，看板和历史里都不再有</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,27 +1471,27 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>F6</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>全选删除</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>历史弹窗勾选若干条（或勾「全选」）→ 点「删除选中」→ 确认</t>
+          <t>编辑里把标签、截止时间清空 → 保存</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>选中的条目全部消失</t>
+          <t>卡片上的标签、截止提示消失</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,27 +1508,27 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>编辑字段</t>
+          <t>打开项目文件夹</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「编辑」→ 改标题/描述/标签 → 保存</t>
+          <t>抽屉里 workspace 行点文件夹图标</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>卡片内容更新</t>
+          <t>服务器那台电脑弹出访达/资源管理器定位到该文件夹</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>编辑弹窗把「状态」从待处理改成等你确认 → 保存</t>
+          <t>抽屉里点「删除」→ 确认</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>卡片从看板消失，归档历史里也没有</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,27 +1582,27 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>悬停验收</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>编辑里把标签清空 → 保存</t>
+          <t>悬停等你确认列的卡片</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>卡片上的标签消失</t>
+          <t>卡片底部浮现「验收通过」「退回修改」两个按钮</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,27 +1619,27 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>任意卡片点「删除」→ 确认弹窗</t>
+          <t>点「验收通过」（悬停按钮或抽屉内）</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有；同一任务再删提示不存在</t>
+          <t>卡片从四列消失；设置 → 归档历史里能看到，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,27 +1656,27 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>G5</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t>G. 编辑任务</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>编辑已归档任务</t>
+          <t>退回修改带反馈</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>历史里没有编辑入口</t>
+          <t>抽屉里点「退回修改」→ 填反馈 → 确认退回</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>归档历史只读（符合预期）</t>
+          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8080/api/tasks` 能读到 `reviewFeedback` 字段</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>反馈流转</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1","name":"Alpha"}' http://localhost:8080/api/agents`</t>
+          <t>退回后让 agent 重新 complete（或编辑改状态到等你确认）</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>成功；`curl http://localhost:8080/api/agents` 能看到 a1/Alpha</t>
+          <t>退回反馈被清除，新一轮验收重新开始</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,27 +1730,27 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>主界面无注册入口</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>先上传头像（`curl -F "file=@x.png" http://localhost:8080/api/avatars`），再 POST /api/agents 带 `avatar`</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>之后该 agent 接取的卡片显示新头像</t>
+          <t>页面上**没有** Agent 注册表单；agent 信息只出现在卡片/抽屉里</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,27 +1767,27 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>空名称预配置</t>
+          <t>API 注册并接取</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"id":"a1"}' http://localhost:8080/api/agents`</t>
+          <t>先 `curl -F "file=@头像.png" .../api/avatars` 记 path，再 `curl -X POST -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;path&gt;"}' .../api/tasks/&lt;id&gt;/claim`</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>名称自动等于 id</t>
+          <t>返回 200，卡片移到处理中列，右上角显示头像</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,27 +1804,27 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>H4</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t>H. Agent 身份（API 预配置）</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>界面不显示 agentId</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>预配置后，该 agent claim 时带别的名称/头像</t>
+          <t>看卡片与抽屉</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>卡片仍显示预配置的名称和头像（不被 agent 覆盖）</t>
+          <t>只显示头像 + 名称，**不显示** agentId（仅存在于 API 层）</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,27 +1841,27 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>回收孤儿任务</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片点「编辑」→ 状态改为「待处理」→ 保存（或 `curl -X POST http://localhost:8080/api/tasks/&lt;id&gt;/recycle`）</t>
+          <t>claim 缺 `name`、头像用字母/emoji、或伪造 `/api/avatars/xxx.png`</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>卡片回到**待处理**列，agent 头像消失</t>
+          <t>返回 422，任务不被接取</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,27 +1878,27 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>回收后再点「接取」</t>
+          <t>两个不同 agentId 先后 claim 同一任务</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>**只有一个成功**，另一个 409</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,27 +1915,27 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
         </is>
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>疑似卡住标记</t>
+          <t>无 agent 操作按钮</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片超过 24 小时未更新（快速验证：把 `internal/webui/app.js` 里 `STUCK_THRESHOLD_MS` 临时改成 `60000` 重启，等 1 分钟）</t>
+          <t>看处理中/遇到阻碍列卡片与抽屉</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>卡片红框 + 红色「疑似卡住」闪烁标记</t>
+          <t>没有「阻碍/完成/解除阻碍」按钮（这些是 agent 的 API 动作）</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,27 +1952,27 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
         </is>
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>API 状态流转</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>卡片在列间正确移动</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,27 +1989,27 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>block 带原因</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -H "Content-Type: application/json" -d '{"title":"API 测试","workspacePath":"C:/x"}' http://localhost:8080/api/tasks`</t>
+          <t>`curl -X POST -d '{"reason":"等 token"}' .../block`</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>卡片与抽屉显示该原因；unblock 后消失</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,27 +2026,27 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>抽屉回收</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim（`curl -X POST -d '{"agentId":"a1"}' http://localhost:8080/api/tasks/&lt;id&gt;/claim`）</t>
+          <t>处理中卡片打开抽屉 →「回收到待处理」</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409 + error 信息</t>
+          <t>卡片回到待处理列，agent 头像消失</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="0">
@@ -2063,27 +2063,27 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C55" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D55" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/tasks?status=archived"`</t>
+          <t>回收后由 agent 重新 claim</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="0">
         <is>
-          <t>返回已归档任务数组，含 `completedAt`</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="0">
@@ -2100,27 +2100,27 @@
     <row r="56">
       <c r="A56" t="inlineStr" s="0">
         <is>
-          <t>J5</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="0">
         <is>
-          <t>J. API 抽查（可选，用命令行）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C56" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>API 回收</t>
         </is>
       </c>
       <c r="D56" t="inlineStr" s="0">
         <is>
-          <t>`curl "http://localhost:8080/api/fs/dirs?path=C%3A%5C"`（Mac 用 `?path=%2F`）</t>
+          <t>`curl -X POST .../api/tasks/&lt;id&gt;/recycle`</t>
         </is>
       </c>
       <c r="E56" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>同样回到待处理</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="0">
@@ -2137,27 +2137,27 @@
     <row r="57">
       <c r="A57" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. 归档历史</t>
         </is>
       </c>
       <c r="C57" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>入口位置</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-arm64`：`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>看顶栏</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>顶栏没有「归档历史」主按钮；在设置（齿轮）菜单里打开</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="0">
@@ -2174,27 +2174,27 @@
     <row r="58">
       <c r="A58" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. 归档历史</t>
         </is>
       </c>
       <c r="C58" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D58" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>打开归档历史</t>
         </is>
       </c>
       <c r="E58" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>显示标题、workspace、标签、完成时间</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="0">
@@ -2211,27 +2211,27 @@
     <row r="59">
       <c r="A59" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="0">
         <is>
-          <t>K. 跨平台（Mac）</t>
+          <t>J. 归档历史</t>
         </is>
       </c>
       <c r="C59" t="inlineStr" s="0">
         <is>
-          <t>Gatekeeper</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D59" t="inlineStr" s="0">
         <is>
-          <t>首次运行若提示"无法验证开发者"</t>
+          <t>点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E59" t="inlineStr" s="0">
         <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+          <t>该条消失</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="0">
@@ -2248,35 +2248,664 @@
     <row r="60">
       <c r="A60" t="inlineStr" s="0">
         <is>
+          <t>J4</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr" s="0">
+        <is>
+          <t>J. 归档历史</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr" s="0">
+        <is>
+          <t>全选删除</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr" s="0">
+        <is>
+          <t>勾选若干条（或全选）→「删除选中」→ 确认</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr" s="0">
+        <is>
+          <t>选中条目全部消失</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr" s="0">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr" s="0">
+        <is>
+          <t>K. 搜索与筛选</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr" s="0">
+        <is>
+          <t>搜索标题</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr" s="0">
+        <is>
+          <t>顶栏搜索框输入标题关键词</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr" s="0">
+        <is>
+          <t>看板就地过滤，四列结构保持</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr" s="0">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr" s="0">
+        <is>
+          <t>K. 搜索与筛选</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr" s="0">
+        <is>
+          <t>搜索 workspace</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr" s="0">
+        <is>
+          <t>输入文件夹名（如 light-kanban）</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr" s="0">
+        <is>
+          <t>该 workspace 的任务被筛出（全路径与简称都能命中）</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr" s="0">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr" s="0">
+        <is>
+          <t>K. 搜索与筛选</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr" s="0">
+        <is>
+          <t>搜索 Agent</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr" s="0">
+        <is>
+          <t>输入 agent 名称</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr" s="0">
+        <is>
+          <t>该 agent 持有的任务被筛出</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr" s="0">
+        <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr" s="0">
-        <is>
-          <t>K. 跨平台（Mac）</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr" s="0">
+      <c r="B64" t="inlineStr" s="0">
+        <is>
+          <t>K. 搜索与筛选</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr" s="0">
+        <is>
+          <t>组合筛选</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr" s="0">
+        <is>
+          <t>筛选里勾 Workspace=light-kanban + 标签=ui</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr" s="0">
+        <is>
+          <t>看板只显示同时匹配的任务，筛选按钮显示激活数量</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr" s="0">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr" s="0">
+        <is>
+          <t>K. 搜索与筛选</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr" s="0">
+        <is>
+          <t>清除筛选</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr" s="0">
+        <is>
+          <t>点「清除全部」</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr" s="0">
+        <is>
+          <t>看板恢复完整</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr" s="0">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr" s="0">
+        <is>
+          <t>L. Agent 预配置（API）</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr" s="0">
+        <is>
+          <t>预配置 agent</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr" s="0">
+        <is>
+          <t>`curl -X POST -d '{"id":"a1","name":"Alpha"}' .../api/agents`</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr" s="0">
+        <is>
+          <t>成功；`curl .../api/agents` 能看到</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr" s="0">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr" s="0">
+        <is>
+          <t>L. Agent 预配置（API）</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr" s="0">
+        <is>
+          <t>更新头像</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr" s="0">
+        <is>
+          <t>上传头像后 POST /api/agents 带 `avatar`</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr" s="0">
+        <is>
+          <t>之后该 agent 接取的卡片显示新头像</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr" s="0">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr" s="0">
+        <is>
+          <t>L. Agent 预配置（API）</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr" s="0">
+        <is>
+          <t>身份钉死</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr" s="0">
+        <is>
+          <t>预配置后该 agent claim 时带别的名称/头像</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr" s="0">
+        <is>
+          <t>卡片仍显示预配置的名称和头像</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr" s="0">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr" s="0">
+        <is>
+          <t>M. API 抽查（可选，用命令行）</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr" s="0">
+        <is>
+          <t>健康检查</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr" s="0">
+        <is>
+          <t>`curl http://localhost:8080/api/health`</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr" s="0">
+        <is>
+          <t>`{"db":"ok","status":"ok"}`</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr" s="0">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr" s="0">
+        <is>
+          <t>M. API 抽查（可选，用命令行）</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="0">
+        <is>
+          <t>创建任务</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr" s="0">
+        <is>
+          <t>`curl -X POST -d '{"title":"API 测试","workspacePath":"/tmp/x"}' .../api/tasks`</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr" s="0">
+        <is>
+          <t>返回任务 JSON，`"status":"todo"`</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr" s="0">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr" s="0">
+        <is>
+          <t>M. API 抽查（可选，用命令行）</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr" s="0">
+        <is>
+          <t>接取冲突</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr" s="0">
+        <is>
+          <t>对同一任务连发两次 claim</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr" s="0">
+        <is>
+          <t>第一次 200，第二次 409</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr" s="0">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr" s="0">
+        <is>
+          <t>M. API 抽查（可选，用命令行）</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr" s="0">
+        <is>
+          <t>归档历史查询</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr" s="0">
+        <is>
+          <t>`curl ".../api/tasks?status=archived"`</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr" s="0">
+        <is>
+          <t>返回已归档数组，含 `completedAt`</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr" s="0">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr" s="0">
+        <is>
+          <t>M. API 抽查（可选，用命令行）</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr" s="0">
+        <is>
+          <t>目录浏览</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr" s="0">
+        <is>
+          <t>`curl ".../api/fs/dirs?path=%2F"`（Mac）</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr" s="0">
+        <is>
+          <t>返回该目录下的子文件夹列表</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr" s="0">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr" s="0">
+        <is>
+          <t>N. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr" s="0">
+        <is>
+          <t>Apple Silicon</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr" s="0">
+        <is>
+          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr" s="0">
+        <is>
+          <t>正常启动，页面功能同 Windows</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr" s="0">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr" s="0">
+        <is>
+          <t>N. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr" s="0">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr" s="0">
+        <is>
+          <t>N. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr" s="0">
+        <is>
+          <t>Gatekeeper</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr" s="0">
+        <is>
+          <t>首次运行若提示"无法验证开发者"</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr" s="0">
+        <is>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr" s="0">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr" s="0">
+        <is>
+          <t>N. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="0">
         <is>
           <t>系统选择</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr" s="0">
+      <c r="D77" t="inlineStr" s="0">
         <is>
           <t>Mac 上点「系统选择…」</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr" s="0">
+      <c r="E77" t="inlineStr" s="0">
         <is>
           <t>弹出 macOS 的 `choose folder` 对话框</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr" s="0">
+      <c r="F77" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2284,7 +2913,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F60">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F77">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(fs): drop native folder picker, browse-only workspace selection
The native system picker (osascript/PowerShell/zenity) hangs or fails when
the server runs without a GUI session, and the in-page browser already
covers the same job — one entry point is enough.

- remove POST /api/fs/pick (+ pickDir machinery and pick_test.go)
- FolderBrowserDialog loses the '系统选择…' button; i18n keys and guide
  copy updated in zh/en
- seed-demo: real product icons for Codex / Claude Code avatars were
  already enforced (spec icon convention); demo workspaces are now
  mkdir -p'd so 'open project folder' never 404s on fresh machines
- docs synced: README x2, AGENTS, PROGRESS, spec.md, checklist (+xlsx)
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G75"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -768,7 +768,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>B9</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
@@ -778,17 +778,17 @@
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>系统选择</t>
+          <t>取消新建</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>点「系统选择…」</t>
+          <t>打开弹窗后点「取消」/ 点弹窗外 / 按 Esc</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>服务器所在电脑弹出系统文件夹对话框，选完路径自动填入</t>
+          <t>弹窗关闭，没有任务被创建</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,27 +805,27 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>B12</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t>B. 新建任务</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>取消新建</t>
+          <t>四列结构</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>打开弹窗后点「取消」/ 点弹窗外 / 按 Esc</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，没有任务被创建</t>
+          <t>待处理(灰○) / 处理中(黄◐) / 遇到阻碍(红!) / 等你确认(绿✓)，列头右侧有任务计数</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,7 +842,7 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
@@ -852,17 +852,17 @@
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>四列结构</t>
+          <t>列独立滚动</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>灌入演示数据后滚动某一列</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>待处理(灰○) / 处理中(黄◐) / 遇到阻碍(红!) / 等你确认(绿✓)，列头右侧有任务计数</t>
+          <t>每列独立上下滚动，页面整体不随任务增多向下增长</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,7 +879,7 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
@@ -889,17 +889,17 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>列独立滚动</t>
+          <t>列头固定</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>灌入演示数据后滚动某一列</t>
+          <t>列内滚动时看列头</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>每列独立上下滚动，页面整体不随任务增多向下增长</t>
+          <t>列标题、计数、快速新增按钮始终停在列顶</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,7 +916,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
@@ -926,17 +926,17 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>列头固定</t>
+          <t>窄屏横滚</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>列内滚动时看列头</t>
+          <t>把窗口拖窄（&lt; ~1300px）</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>列标题、计数、快速新增按钮始终停在列顶</t>
+          <t>看板出现横向滚动，四列保持原宽度不重排</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,7 +953,7 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>C4</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
@@ -963,17 +963,17 @@
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>窄屏横滚</t>
+          <t>高密度</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>把窗口拖窄（&lt; ~1300px）</t>
+          <t>一屏内数卡片</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>看板出现横向滚动，四列保持原宽度不重排</t>
+          <t>同样屏幕能放下明显比旧版更多的卡片，且不拥挤</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,27 +990,27 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>C5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t>C. 看板布局</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>高密度</t>
+          <t>短号与头像</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>一屏内数卡片</t>
+          <t>看任意卡片第一行</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>同样屏幕能放下明显比旧版更多的卡片，且不拥挤</t>
+          <t>左侧淡灰 `LK-XXXX` 短号，右侧 18px agent 头像（未接取的卡片没有头像）</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,7 +1027,7 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>短号与头像</t>
+          <t>workspace 显示</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>看任意卡片第一行</t>
+          <t>看卡片底部</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>左侧淡灰 `LK-XXXX` 短号，右侧 18px agent 头像（未接取的卡片没有头像）</t>
+          <t>只显示文件夹名（如 light-kanban）+ 颜色点，**不显示**完整路径；悬停可见全路径</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,7 +1064,7 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>workspace 显示</t>
+          <t>标签折叠</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>看卡片底部</t>
+          <t>找一张 3+ 标签的卡</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>只显示文件夹名（如 light-kanban）+ 颜色点，**不显示**完整路径；悬停可见全路径</t>
+          <t>最多 2 个标签 + 「+N」，不撑高卡片</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,7 +1101,7 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>标签折叠</t>
+          <t>截止提示</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>找一张 3+ 标签的卡</t>
+          <t>演示数据里找今天截止 / 已逾期卡片</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>最多 2 个标签 + 「+N」，不撑高卡片</t>
+          <t>分别显示黄色「今天截止」/ 红色「已逾期」；未来截止显示灰色短日期</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,7 +1138,7 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
@@ -1148,17 +1148,17 @@
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>截止提示</t>
+          <t>卡住标记</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>演示数据里找今天截止 / 已逾期卡片</t>
+          <t>处理中超过 24h 未更新的任务</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>分别显示黄色「今天截止」/ 红色「已逾期」；未来截止显示灰色短日期</t>
+          <t>卡片底部出现「⚠ 疑似卡住」，无红框无闪烁</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,7 +1175,7 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>卡住标记</t>
+          <t>阻碍原因</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>处理中超过 24h 未更新的任务</t>
+          <t>看遇到阻碍列卡片</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>卡片底部出现「⚠ 疑似卡住」，无红框无闪烁</t>
+          <t>卡片上直接以红色「! 原因」显示 agent 填的 blockReason</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,7 +1212,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>阻碍原因</t>
+          <t>长标题</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>看遇到阻碍列卡片</t>
+          <t>找一张长标题卡</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>卡片上直接以红色「! 原因」显示 agent 填的 blockReason</t>
+          <t>标题最多两行截断，卡片不被撑爆</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,27 +1249,27 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
         <is>
-          <t>D. 卡片信息</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>长标题</t>
+          <t>打开抽屉</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>找一张长标题卡</t>
+          <t>点任意卡片</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>标题最多两行截断，卡片不被撑爆</t>
+          <t>右侧滑出抽屉，看板仍部分可见；含短号、标题、状态、Agent、workspace、描述、标签、截止、创建/更新时间</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,7 +1286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1296,17 +1296,17 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>打开抽屉</t>
+          <t>关闭抽屉</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>点任意卡片</t>
+          <t>点 × / 点抽屉外 / 按 Esc</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>右侧滑出抽屉，看板仍部分可见；含短号、标题、状态、Agent、workspace、描述、标签、截止、创建/更新时间</t>
+          <t>抽屉关闭，回到原看板位置</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,7 +1323,7 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
@@ -1333,17 +1333,17 @@
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>关闭抽屉</t>
+          <t>查看/编辑分离</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>点 × / 点抽屉外 / 按 Esc</t>
+          <t>打开抽屉</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>抽屉关闭，回到原看板位置</t>
+          <t>默认是查看模式，没有输入框；点「编辑」才进入编辑</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,7 +1360,7 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>E3</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
@@ -1370,17 +1370,17 @@
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>查看/编辑分离</t>
+          <t>编辑保存</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>打开抽屉</t>
+          <t>编辑标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>默认是查看模式，没有输入框；点「编辑」才进入编辑</t>
+          <t>回到查看模式，卡片内容更新</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,7 +1397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>E4</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>编辑保存</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>编辑标题/描述/标签 → 保存</t>
+          <t>编辑里把状态从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>回到查看模式，卡片内容更新</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,7 +1434,7 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>E5</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>编辑里把状态从待处理改成等你确认 → 保存</t>
+          <t>编辑里把标签、截止时间清空 → 保存</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>卡片上的标签、截止提示消失</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,7 +1471,7 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>E6</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>打开项目文件夹</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>编辑里把标签、截止时间清空 → 保存</t>
+          <t>抽屉里 workspace 行点文件夹图标</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>卡片上的标签、截止提示消失</t>
+          <t>服务器那台电脑弹出访达/资源管理器定位到该文件夹</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,7 +1508,7 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>E7</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>打开项目文件夹</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>抽屉里 workspace 行点文件夹图标</t>
+          <t>抽屉里点「删除」→ 确认</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>服务器那台电脑弹出访达/资源管理器定位到该文件夹</t>
+          <t>卡片从看板消失，归档历史里也没有</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>E8</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>E. 任务抽屉</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>悬停验收</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>抽屉里点「删除」→ 确认</t>
+          <t>悬停等你确认列的卡片</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有</t>
+          <t>卡片底部浮现「验收通过」「退回修改」两个按钮</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,7 +1582,7 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>悬停验收</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>悬停等你确认列的卡片</t>
+          <t>点「验收通过」（悬停按钮或抽屉内）</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>卡片底部浮现「验收通过」「退回修改」两个按钮</t>
+          <t>卡片从四列消失；设置 → 归档历史里能看到，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,7 +1619,7 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
@@ -1629,17 +1629,17 @@
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>退回修改带反馈</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>点「验收通过」（悬停按钮或抽屉内）</t>
+          <t>抽屉里点「退回修改」→ 填反馈 → 确认退回</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；设置 → 归档历史里能看到，带「完成于 …」时间</t>
+          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8080/api/tasks` 能读到 `reviewFeedback` 字段</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,7 +1656,7 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
@@ -1666,17 +1666,17 @@
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>退回修改带反馈</t>
+          <t>反馈流转</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>抽屉里点「退回修改」→ 填反馈 → 确认退回</t>
+          <t>退回后让 agent 重新 complete（或编辑改状态到等你确认）</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8080/api/tasks` 能读到 `reviewFeedback` 字段</t>
+          <t>退回反馈被清除，新一轮验收重新开始</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>反馈流转</t>
+          <t>主界面无注册入口</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>退回后让 agent 重新 complete（或编辑改状态到等你确认）</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>退回反馈被清除，新一轮验收重新开始</t>
+          <t>页面上**没有** Agent 注册表单；agent 信息只出现在卡片/抽屉里</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,7 +1730,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>主界面无注册入口</t>
+          <t>API 注册并接取</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>先 `curl -F "file=@头像.png" .../api/avatars` 记 path，再 `curl -X POST -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;path&gt;"}' .../api/tasks/&lt;id&gt;/claim`</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>页面上**没有** Agent 注册表单；agent 信息只出现在卡片/抽屉里</t>
+          <t>返回 200，卡片移到处理中列，右上角显示头像</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,7 +1767,7 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
@@ -1777,17 +1777,17 @@
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>API 注册并接取</t>
+          <t>界面不显示 agentId</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>先 `curl -F "file=@头像.png" .../api/avatars` 记 path，再 `curl -X POST -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;path&gt;"}' .../api/tasks/&lt;id&gt;/claim`</t>
+          <t>看卡片与抽屉</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>返回 200，卡片移到处理中列，右上角显示头像</t>
+          <t>只显示头像 + 名称，**不显示** agentId（仅存在于 API 层）</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,7 +1804,7 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
@@ -1814,17 +1814,17 @@
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>界面不显示 agentId</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>看卡片与抽屉</t>
+          <t>claim 缺 `name`、头像用字母/emoji、或伪造 `/api/avatars/xxx.png`</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>只显示头像 + 名称，**不显示** agentId（仅存在于 API 层）</t>
+          <t>返回 422，任务不被接取</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,7 +1841,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>缺名称/头像被拒</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>claim 缺 `name`、头像用字母/emoji、或伪造 `/api/avatars/xxx.png`</t>
+          <t>两个不同 agentId 先后 claim 同一任务</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>返回 422，任务不被接取</t>
+          <t>**只有一个成功**，另一个 409</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,27 +1878,27 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>G5</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
         <is>
-          <t>G. 接取任务 &amp; agent 身份（API）</t>
+          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>无 agent 操作按钮</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>两个不同 agentId 先后 claim 同一任务</t>
+          <t>看处理中/遇到阻碍列卡片与抽屉</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>**只有一个成功**，另一个 409</t>
+          <t>没有「阻碍/完成/解除阻碍」按钮（这些是 agent 的 API 动作）</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,7 +1915,7 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>无 agent 操作按钮</t>
+          <t>API 状态流转</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>看处理中/遇到阻碍列卡片与抽屉</t>
+          <t>curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>没有「阻碍/完成/解除阻碍」按钮（这些是 agent 的 API 动作）</t>
+          <t>卡片在列间正确移动</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,7 +1952,7 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>API 状态流转</t>
+          <t>block 带原因</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
+          <t>`curl -X POST -d '{"reason":"等 token"}' .../block`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>卡片在列间正确移动</t>
+          <t>卡片与抽屉显示该原因；unblock 后消失</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,27 +1989,27 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>block 带原因</t>
+          <t>抽屉回收</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -d '{"reason":"等 token"}' .../block`</t>
+          <t>处理中卡片打开抽屉 →「回收到待处理」</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>卡片与抽屉显示该原因；unblock 后消失</t>
+          <t>卡片回到待处理列，agent 头像消失</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,7 +2026,7 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t>抽屉回收</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片打开抽屉 →「回收到待处理」</t>
+          <t>回收后由 agent 重新 claim</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="0">
         <is>
-          <t>卡片回到待处理列，agent 头像消失</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="0">
@@ -2063,7 +2063,7 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="0">
@@ -2073,17 +2073,17 @@
       </c>
       <c r="C55" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>API 回收</t>
         </is>
       </c>
       <c r="D55" t="inlineStr" s="0">
         <is>
-          <t>回收后由 agent 重新 claim</t>
+          <t>`curl -X POST .../api/tasks/&lt;id&gt;/recycle`</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>同样回到待处理</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="0">
@@ -2100,27 +2100,27 @@
     <row r="56">
       <c r="A56" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>J. 归档历史</t>
         </is>
       </c>
       <c r="C56" t="inlineStr" s="0">
         <is>
-          <t>API 回收</t>
+          <t>入口位置</t>
         </is>
       </c>
       <c r="D56" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST .../api/tasks/&lt;id&gt;/recycle`</t>
+          <t>看顶栏</t>
         </is>
       </c>
       <c r="E56" t="inlineStr" s="0">
         <is>
-          <t>同样回到待处理</t>
+          <t>顶栏没有「归档历史」主按钮；在设置（齿轮）菜单里打开</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="0">
@@ -2137,7 +2137,7 @@
     <row r="57">
       <c r="A57" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="0">
@@ -2147,17 +2147,17 @@
       </c>
       <c r="C57" t="inlineStr" s="0">
         <is>
-          <t>入口位置</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="0">
         <is>
-          <t>看顶栏</t>
+          <t>打开归档历史</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="0">
         <is>
-          <t>顶栏没有「归档历史」主按钮；在设置（齿轮）菜单里打开</t>
+          <t>显示标题、workspace、标签、完成时间</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="0">
@@ -2174,7 +2174,7 @@
     <row r="58">
       <c r="A58" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="0">
@@ -2184,17 +2184,17 @@
       </c>
       <c r="C58" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D58" t="inlineStr" s="0">
         <is>
-          <t>打开归档历史</t>
+          <t>点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E58" t="inlineStr" s="0">
         <is>
-          <t>显示标题、workspace、标签、完成时间</t>
+          <t>该条消失</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="0">
@@ -2211,7 +2211,7 @@
     <row r="59">
       <c r="A59" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="0">
@@ -2221,17 +2221,17 @@
       </c>
       <c r="C59" t="inlineStr" s="0">
         <is>
-          <t>单条删除</t>
+          <t>全选删除</t>
         </is>
       </c>
       <c r="D59" t="inlineStr" s="0">
         <is>
-          <t>点某条「删除」→ 确认</t>
+          <t>勾选若干条（或全选）→「删除选中」→ 确认</t>
         </is>
       </c>
       <c r="E59" t="inlineStr" s="0">
         <is>
-          <t>该条消失</t>
+          <t>选中条目全部消失</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="0">
@@ -2248,27 +2248,27 @@
     <row r="60">
       <c r="A60" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr" s="0">
         <is>
-          <t>J. 归档历史</t>
+          <t>K. 搜索与筛选</t>
         </is>
       </c>
       <c r="C60" t="inlineStr" s="0">
         <is>
-          <t>全选删除</t>
+          <t>搜索标题</t>
         </is>
       </c>
       <c r="D60" t="inlineStr" s="0">
         <is>
-          <t>勾选若干条（或全选）→「删除选中」→ 确认</t>
+          <t>顶栏搜索框输入标题关键词</t>
         </is>
       </c>
       <c r="E60" t="inlineStr" s="0">
         <is>
-          <t>选中条目全部消失</t>
+          <t>看板就地过滤，四列结构保持</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="0">
@@ -2285,7 +2285,7 @@
     <row r="61">
       <c r="A61" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B61" t="inlineStr" s="0">
@@ -2295,17 +2295,17 @@
       </c>
       <c r="C61" t="inlineStr" s="0">
         <is>
-          <t>搜索标题</t>
+          <t>搜索 workspace</t>
         </is>
       </c>
       <c r="D61" t="inlineStr" s="0">
         <is>
-          <t>顶栏搜索框输入标题关键词</t>
+          <t>输入文件夹名（如 light-kanban）</t>
         </is>
       </c>
       <c r="E61" t="inlineStr" s="0">
         <is>
-          <t>看板就地过滤，四列结构保持</t>
+          <t>该 workspace 的任务被筛出（全路径与简称都能命中）</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="0">
@@ -2322,7 +2322,7 @@
     <row r="62">
       <c r="A62" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr" s="0">
@@ -2332,17 +2332,17 @@
       </c>
       <c r="C62" t="inlineStr" s="0">
         <is>
-          <t>搜索 workspace</t>
+          <t>搜索 Agent</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="0">
         <is>
-          <t>输入文件夹名（如 light-kanban）</t>
+          <t>输入 agent 名称</t>
         </is>
       </c>
       <c r="E62" t="inlineStr" s="0">
         <is>
-          <t>该 workspace 的任务被筛出（全路径与简称都能命中）</t>
+          <t>该 agent 持有的任务被筛出</t>
         </is>
       </c>
       <c r="F62" t="inlineStr" s="0">
@@ -2359,7 +2359,7 @@
     <row r="63">
       <c r="A63" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="B63" t="inlineStr" s="0">
@@ -2369,17 +2369,17 @@
       </c>
       <c r="C63" t="inlineStr" s="0">
         <is>
-          <t>搜索 Agent</t>
+          <t>组合筛选</t>
         </is>
       </c>
       <c r="D63" t="inlineStr" s="0">
         <is>
-          <t>输入 agent 名称</t>
+          <t>筛选里勾 Workspace=light-kanban + 标签=ui</t>
         </is>
       </c>
       <c r="E63" t="inlineStr" s="0">
         <is>
-          <t>该 agent 持有的任务被筛出</t>
+          <t>看板只显示同时匹配的任务，筛选按钮显示激活数量</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="0">
@@ -2396,7 +2396,7 @@
     <row r="64">
       <c r="A64" t="inlineStr" s="0">
         <is>
-          <t>K4</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="B64" t="inlineStr" s="0">
@@ -2406,17 +2406,17 @@
       </c>
       <c r="C64" t="inlineStr" s="0">
         <is>
-          <t>组合筛选</t>
+          <t>清除筛选</t>
         </is>
       </c>
       <c r="D64" t="inlineStr" s="0">
         <is>
-          <t>筛选里勾 Workspace=light-kanban + 标签=ui</t>
+          <t>点「清除全部」</t>
         </is>
       </c>
       <c r="E64" t="inlineStr" s="0">
         <is>
-          <t>看板只显示同时匹配的任务，筛选按钮显示激活数量</t>
+          <t>看板恢复完整</t>
         </is>
       </c>
       <c r="F64" t="inlineStr" s="0">
@@ -2433,27 +2433,27 @@
     <row r="65">
       <c r="A65" t="inlineStr" s="0">
         <is>
-          <t>K5</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr" s="0">
         <is>
-          <t>K. 搜索与筛选</t>
+          <t>L. Agent 预配置（API）</t>
         </is>
       </c>
       <c r="C65" t="inlineStr" s="0">
         <is>
-          <t>清除筛选</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D65" t="inlineStr" s="0">
         <is>
-          <t>点「清除全部」</t>
+          <t>`curl -X POST -d '{"id":"a1","name":"Alpha"}' .../api/agents`</t>
         </is>
       </c>
       <c r="E65" t="inlineStr" s="0">
         <is>
-          <t>看板恢复完整</t>
+          <t>成功；`curl .../api/agents` 能看到</t>
         </is>
       </c>
       <c r="F65" t="inlineStr" s="0">
@@ -2470,7 +2470,7 @@
     <row r="66">
       <c r="A66" t="inlineStr" s="0">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr" s="0">
@@ -2480,17 +2480,17 @@
       </c>
       <c r="C66" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D66" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -d '{"id":"a1","name":"Alpha"}' .../api/agents`</t>
+          <t>上传头像后 POST /api/agents 带 `avatar`</t>
         </is>
       </c>
       <c r="E66" t="inlineStr" s="0">
         <is>
-          <t>成功；`curl .../api/agents` 能看到</t>
+          <t>之后该 agent 接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F66" t="inlineStr" s="0">
@@ -2507,7 +2507,7 @@
     <row r="67">
       <c r="A67" t="inlineStr" s="0">
         <is>
-          <t>L2</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr" s="0">
@@ -2517,17 +2517,17 @@
       </c>
       <c r="C67" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D67" t="inlineStr" s="0">
         <is>
-          <t>上传头像后 POST /api/agents 带 `avatar`</t>
+          <t>预配置后该 agent claim 时带别的名称/头像</t>
         </is>
       </c>
       <c r="E67" t="inlineStr" s="0">
         <is>
-          <t>之后该 agent 接取的卡片显示新头像</t>
+          <t>卡片仍显示预配置的名称和头像</t>
         </is>
       </c>
       <c r="F67" t="inlineStr" s="0">
@@ -2544,27 +2544,27 @@
     <row r="68">
       <c r="A68" t="inlineStr" s="0">
         <is>
-          <t>L3</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr" s="0">
         <is>
-          <t>L. Agent 预配置（API）</t>
+          <t>M. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C68" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D68" t="inlineStr" s="0">
         <is>
-          <t>预配置后该 agent claim 时带别的名称/头像</t>
+          <t>`curl http://localhost:8080/api/health`</t>
         </is>
       </c>
       <c r="E68" t="inlineStr" s="0">
         <is>
-          <t>卡片仍显示预配置的名称和头像</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F68" t="inlineStr" s="0">
@@ -2581,7 +2581,7 @@
     <row r="69">
       <c r="A69" t="inlineStr" s="0">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B69" t="inlineStr" s="0">
@@ -2591,17 +2591,17 @@
       </c>
       <c r="C69" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D69" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>`curl -X POST -d '{"title":"API 测试","workspacePath":"/tmp/x"}' .../api/tasks`</t>
         </is>
       </c>
       <c r="E69" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="0">
@@ -2618,7 +2618,7 @@
     <row r="70">
       <c r="A70" t="inlineStr" s="0">
         <is>
-          <t>M2</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B70" t="inlineStr" s="0">
@@ -2628,17 +2628,17 @@
       </c>
       <c r="C70" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D70" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -d '{"title":"API 测试","workspacePath":"/tmp/x"}' .../api/tasks`</t>
+          <t>对同一任务连发两次 claim</t>
         </is>
       </c>
       <c r="E70" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>第一次 200，第二次 409</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="0">
@@ -2655,7 +2655,7 @@
     <row r="71">
       <c r="A71" t="inlineStr" s="0">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B71" t="inlineStr" s="0">
@@ -2665,17 +2665,17 @@
       </c>
       <c r="C71" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D71" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim</t>
+          <t>`curl ".../api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409</t>
+          <t>返回已归档数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="0">
@@ -2692,7 +2692,7 @@
     <row r="72">
       <c r="A72" t="inlineStr" s="0">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B72" t="inlineStr" s="0">
@@ -2702,17 +2702,17 @@
       </c>
       <c r="C72" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D72" t="inlineStr" s="0">
         <is>
-          <t>`curl ".../api/tasks?status=archived"`</t>
+          <t>`curl ".../api/fs/dirs?path=%2F"`（Mac）</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="0">
         <is>
-          <t>返回已归档数组，含 `completedAt`</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="0">
@@ -2729,27 +2729,27 @@
     <row r="73">
       <c r="A73" t="inlineStr" s="0">
         <is>
-          <t>M5</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr" s="0">
         <is>
-          <t>M. API 抽查（可选，用命令行）</t>
+          <t>N. 跨平台（Mac）</t>
         </is>
       </c>
       <c r="C73" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="0">
         <is>
-          <t>`curl ".../api/fs/dirs?path=%2F"`（Mac）</t>
+          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="0">
@@ -2766,7 +2766,7 @@
     <row r="74">
       <c r="A74" t="inlineStr" s="0">
         <is>
-          <t>N1</t>
+          <t>N2</t>
         </is>
       </c>
       <c r="B74" t="inlineStr" s="0">
@@ -2776,17 +2776,17 @@
       </c>
       <c r="C74" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>Intel Mac</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="0">
         <is>
-          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="0">
@@ -2803,7 +2803,7 @@
     <row r="75">
       <c r="A75" t="inlineStr" s="0">
         <is>
-          <t>N2</t>
+          <t>N3</t>
         </is>
       </c>
       <c r="B75" t="inlineStr" s="0">
@@ -2813,17 +2813,17 @@
       </c>
       <c r="C75" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>Gatekeeper</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>首次运行若提示"无法验证开发者"</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="0">
@@ -2832,80 +2832,6 @@
         </is>
       </c>
       <c r="G75" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr" s="0">
-        <is>
-          <t>N3</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr" s="0">
-        <is>
-          <t>N. 跨平台（Mac）</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr" s="0">
-        <is>
-          <t>Gatekeeper</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr" s="0">
-        <is>
-          <t>首次运行若提示"无法验证开发者"</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr" s="0">
-        <is>
-          <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr" s="0">
-        <is>
-          <t>N4</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr" s="0">
-        <is>
-          <t>N. 跨平台（Mac）</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr" s="0">
-        <is>
-          <t>系统选择</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr" s="0">
-        <is>
-          <t>Mac 上点「系统选择…」</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr" s="0">
-        <is>
-          <t>弹出 macOS 的 `choose folder` 对话框</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2913,7 +2839,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F77">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F75">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(fs): native folder picker replaces in-page browse; default port :8641
Per acceptance feedback:
- restore POST /api/fs/pick (native OS dialog); on macOS the dialog now
  self-activates ('tell me to activate') so it pops in front — the old
  'hang' was a hidden dialog waiting for an answer, not a crash
- workspace path is directly editable (type/paste) in the task form;
  while the system dialog is open the button offers 'stop waiting'
  (aborts the request, server stops waiting too)
- remove GET /api/fs/dirs, the in-page FolderBrowser dialog and its
  styles/utils/i18n keys — one folder-picking way, not two
- default listen port 8080 -> 8641 (less collision-prone); docs, vite
  proxy, Makefile, seed script and checklist updated accordingly
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -117,12 +117,12 @@
       </c>
       <c r="D2" t="inlineStr" s="0">
         <is>
-          <t>运行 `./dist/light-kanban -addr :8080`</t>
+          <t>运行 `./dist/light-kanban -addr :8641`</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>命令行出现 `listening on :8080`，不报错</t>
+          <t>命令行出现 `listening on :8641`，不报错</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -159,7 +159,7 @@
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>弹出控制台窗口并**自动打开浏览器** http://localhost:8080</t>
+          <t>弹出控制台窗口并**自动打开浏览器** http://localhost:8641</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
@@ -191,7 +191,7 @@
       </c>
       <c r="D4" t="inlineStr" s="0">
         <is>
-          <t>浏览器开 http://localhost:8080/api/health</t>
+          <t>浏览器开 http://localhost:8641/api/health</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="0">
@@ -228,7 +228,7 @@
       </c>
       <c r="D5" t="inlineStr" s="0">
         <is>
-          <t>打开 http://localhost:8080</t>
+          <t>打开 http://localhost:8641</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="0">
@@ -704,17 +704,17 @@
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t>页内浏览选目录</t>
+          <t>直接输入路径</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>点路径框旁「浏览…」→ 点进文件夹 →「选择此文件夹」</t>
+          <t>在 workspace 路径框手动输入/粘贴一个存在的绝对路径</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>路径框自动填入所选文件夹完整路径</t>
+          <t>正常创建任务，卡片显示路径末级名称</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
@@ -741,17 +741,17 @@
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>浏览上级</t>
+          <t>系统选择</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
         <is>
-          <t>浏览弹窗里点「上级」</t>
+          <t>点路径框旁「选择…」</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>回到上一级目录；到根目录后 Mac 显示 `/`</t>
+          <t>运行看板的电脑弹出系统文件夹窗口并置前；选完自动填入路径；点「取消等待」可中止</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8080/api/tasks` 能读到 `reviewFeedback` 字段</t>
+          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8641/api/tasks` 能读到 `reviewFeedback` 字段</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="D68" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8080/api/health`</t>
+          <t>`curl http://localhost:8641/api/health`</t>
         </is>
       </c>
       <c r="E68" t="inlineStr" s="0">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="D73" t="inlineStr" s="0">
         <is>
-          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8080`</t>
+          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8641`</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="0">

</xml_diff>

<commit_message>
feat(ui): picker failure alert now guides manual path entry
When the native picker cannot run (headless server, SSH, no zenity/
kdialog), the error alert explains the recovery path: type or paste an
absolute path directly. Checklist gains row B8b for the fallback case.
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -768,7 +768,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>B12</t>
+          <t>B8b</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
@@ -778,17 +778,17 @@
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t>取消新建</t>
+          <t>系统选择失败兜底</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>打开弹窗后点「取消」/ 点弹窗外 / 按 Esc</t>
+          <t>无桌面环境（如 SSH）下点「选择…」</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>弹窗关闭，没有任务被创建</t>
+          <t>提示失败原因，并引导直接在输入框输入/粘贴绝对路径；手动输入后任务可正常创建</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -805,27 +805,27 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>C1</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t>C. 看板布局</t>
+          <t>B. 新建任务</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t>四列结构</t>
+          <t>取消新建</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>打开弹窗后点「取消」/ 点弹窗外 / 按 Esc</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>待处理(灰○) / 处理中(黄◐) / 遇到阻碍(红!) / 等你确认(绿✓)，列头右侧有任务计数</t>
+          <t>弹窗关闭，没有任务被创建</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
@@ -842,7 +842,7 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
@@ -852,17 +852,17 @@
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t>列独立滚动</t>
+          <t>四列结构</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
         <is>
-          <t>灌入演示数据后滚动某一列</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>每列独立上下滚动，页面整体不随任务增多向下增长</t>
+          <t>待处理(灰○) / 处理中(黄◐) / 遇到阻碍(红!) / 等你确认(绿✓)，列头右侧有任务计数</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
@@ -879,7 +879,7 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
@@ -889,17 +889,17 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t>列头固定</t>
+          <t>列独立滚动</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>列内滚动时看列头</t>
+          <t>灌入演示数据后滚动某一列</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>列标题、计数、快速新增按钮始终停在列顶</t>
+          <t>每列独立上下滚动，页面整体不随任务增多向下增长</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
@@ -916,7 +916,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
@@ -926,17 +926,17 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>窄屏横滚</t>
+          <t>列头固定</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>把窗口拖窄（&lt; ~1300px）</t>
+          <t>列内滚动时看列头</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>看板出现横向滚动，四列保持原宽度不重排</t>
+          <t>列标题、计数、快速新增按钮始终停在列顶</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
@@ -953,7 +953,7 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>C5</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
@@ -963,17 +963,17 @@
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t>高密度</t>
+          <t>窄屏横滚</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>一屏内数卡片</t>
+          <t>把窗口拖窄（&lt; ~1300px）</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>同样屏幕能放下明显比旧版更多的卡片，且不拥挤</t>
+          <t>看板出现横向滚动，四列保持原宽度不重排</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
@@ -990,27 +990,27 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>D1</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t>D. 卡片信息</t>
+          <t>C. 看板布局</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t>短号与头像</t>
+          <t>高密度</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
         <is>
-          <t>看任意卡片第一行</t>
+          <t>一屏内数卡片</t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>左侧淡灰 `LK-XXXX` 短号，右侧 18px agent 头像（未接取的卡片没有头像）</t>
+          <t>同样屏幕能放下明显比旧版更多的卡片，且不拥挤</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
@@ -1027,7 +1027,7 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t>workspace 显示</t>
+          <t>短号与头像</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
         <is>
-          <t>看卡片底部</t>
+          <t>看任意卡片第一行</t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>只显示文件夹名（如 light-kanban）+ 颜色点，**不显示**完整路径；悬停可见全路径</t>
+          <t>左侧淡灰 `LK-XXXX` 短号，右侧 18px agent 头像（未接取的卡片没有头像）</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1064,7 +1064,7 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t>标签折叠</t>
+          <t>workspace 显示</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
         <is>
-          <t>找一张 3+ 标签的卡</t>
+          <t>看卡片底部</t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>最多 2 个标签 + 「+N」，不撑高卡片</t>
+          <t>只显示文件夹名（如 light-kanban）+ 颜色点，**不显示**完整路径；悬停可见全路径</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
@@ -1101,7 +1101,7 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t>截止提示</t>
+          <t>标签折叠</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
         <is>
-          <t>演示数据里找今天截止 / 已逾期卡片</t>
+          <t>找一张 3+ 标签的卡</t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>分别显示黄色「今天截止」/ 红色「已逾期」；未来截止显示灰色短日期</t>
+          <t>最多 2 个标签 + 「+N」，不撑高卡片</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -1138,7 +1138,7 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
@@ -1148,17 +1148,17 @@
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t>卡住标记</t>
+          <t>截止提示</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
         <is>
-          <t>处理中超过 24h 未更新的任务</t>
+          <t>演示数据里找今天截止 / 已逾期卡片</t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>卡片底部出现「⚠ 疑似卡住」，无红框无闪烁</t>
+          <t>分别显示黄色「今天截止」/ 红色「已逾期」；未来截止显示灰色短日期</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -1175,7 +1175,7 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t>阻碍原因</t>
+          <t>卡住标记</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
         <is>
-          <t>看遇到阻碍列卡片</t>
+          <t>处理中超过 24h 未更新的任务</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>卡片上直接以红色「! 原因」显示 agent 填的 blockReason</t>
+          <t>卡片底部出现「⚠ 疑似卡住」，无红框无闪烁</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -1212,7 +1212,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t>长标题</t>
+          <t>阻碍原因</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
         <is>
-          <t>找一张长标题卡</t>
+          <t>看遇到阻碍列卡片</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>标题最多两行截断，卡片不被撑爆</t>
+          <t>卡片上直接以红色「! 原因」显示 agent 填的 blockReason</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -1249,27 +1249,27 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>E1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
         <is>
-          <t>E. 任务抽屉</t>
+          <t>D. 卡片信息</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t>打开抽屉</t>
+          <t>长标题</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
         <is>
-          <t>点任意卡片</t>
+          <t>找一张长标题卡</t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>右侧滑出抽屉，看板仍部分可见；含短号、标题、状态、Agent、workspace、描述、标签、截止、创建/更新时间</t>
+          <t>标题最多两行截断，卡片不被撑爆</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -1286,7 +1286,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -1296,17 +1296,17 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t>关闭抽屉</t>
+          <t>打开抽屉</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
         <is>
-          <t>点 × / 点抽屉外 / 按 Esc</t>
+          <t>点任意卡片</t>
         </is>
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>抽屉关闭，回到原看板位置</t>
+          <t>右侧滑出抽屉，看板仍部分可见；含短号、标题、状态、Agent、workspace、描述、标签、截止、创建/更新时间</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -1323,7 +1323,7 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>E3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
@@ -1333,17 +1333,17 @@
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t>查看/编辑分离</t>
+          <t>关闭抽屉</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>打开抽屉</t>
+          <t>点 × / 点抽屉外 / 按 Esc</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>默认是查看模式，没有输入框；点「编辑」才进入编辑</t>
+          <t>抽屉关闭，回到原看板位置</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -1360,7 +1360,7 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>E4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
@@ -1370,17 +1370,17 @@
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t>编辑保存</t>
+          <t>查看/编辑分离</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>编辑标题/描述/标签 → 保存</t>
+          <t>打开抽屉</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>回到查看模式，卡片内容更新</t>
+          <t>默认是查看模式，没有输入框；点「编辑」才进入编辑</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -1397,7 +1397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>E5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t>人工纠正状态</t>
+          <t>编辑保存</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
         <is>
-          <t>编辑里把状态从待处理改成等你确认 → 保存</t>
+          <t>编辑标题/描述/标签 → 保存</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>卡片直接移到等你确认列</t>
+          <t>回到查看模式，卡片内容更新</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -1434,7 +1434,7 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>E6</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t>清空可选字段</t>
+          <t>人工纠正状态</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
         <is>
-          <t>编辑里把标签、截止时间清空 → 保存</t>
+          <t>编辑里把状态从待处理改成等你确认 → 保存</t>
         </is>
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>卡片上的标签、截止提示消失</t>
+          <t>卡片直接移到等你确认列</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -1471,7 +1471,7 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t>打开项目文件夹</t>
+          <t>清空可选字段</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
         <is>
-          <t>抽屉里 workspace 行点文件夹图标</t>
+          <t>编辑里把标签、截止时间清空 → 保存</t>
         </is>
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>服务器那台电脑弹出访达/资源管理器定位到该文件夹</t>
+          <t>卡片上的标签、截止提示消失</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
@@ -1508,7 +1508,7 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>E8</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t>删除任务</t>
+          <t>打开项目文件夹</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
         <is>
-          <t>抽屉里点「删除」→ 确认</t>
+          <t>抽屉里 workspace 行点文件夹图标</t>
         </is>
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>卡片从看板消失，归档历史里也没有</t>
+          <t>服务器那台电脑弹出访达/资源管理器定位到该文件夹</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
@@ -1545,27 +1545,27 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>F1</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t>F. 验收（等你确认）</t>
+          <t>E. 任务抽屉</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t>悬停验收</t>
+          <t>删除任务</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
         <is>
-          <t>悬停等你确认列的卡片</t>
+          <t>抽屉里点「删除」→ 确认</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>卡片底部浮现「验收通过」「退回修改」两个按钮</t>
+          <t>卡片从看板消失，归档历史里也没有</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
@@ -1582,7 +1582,7 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>F2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t>验收通过</t>
+          <t>悬停验收</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
         <is>
-          <t>点「验收通过」（悬停按钮或抽屉内）</t>
+          <t>悬停等你确认列的卡片</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>卡片从四列消失；设置 → 归档历史里能看到，带「完成于 …」时间</t>
+          <t>卡片底部浮现「验收通过」「退回修改」两个按钮</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
@@ -1619,7 +1619,7 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>F3</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
@@ -1629,17 +1629,17 @@
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t>退回修改带反馈</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
         <is>
-          <t>抽屉里点「退回修改」→ 填反馈 → 确认退回</t>
+          <t>点「验收通过」（悬停按钮或抽屉内）</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8641/api/tasks` 能读到 `reviewFeedback` 字段</t>
+          <t>卡片从四列消失；设置 → 归档历史里能看到，带「完成于 …」时间</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
@@ -1656,7 +1656,7 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>F4</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
@@ -1666,17 +1666,17 @@
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t>反馈流转</t>
+          <t>退回修改带反馈</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
         <is>
-          <t>退回后让 agent 重新 complete（或编辑改状态到等你确认）</t>
+          <t>抽屉里点「退回修改」→ 填反馈 → 确认退回</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>退回反馈被清除，新一轮验收重新开始</t>
+          <t>卡片回到处理中列；抽屉里可见「退回反馈」；`curl http://localhost:8641/api/tasks` 能读到 `reviewFeedback` 字段</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
@@ -1693,27 +1693,27 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>G1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t>G. 接取任务 &amp; agent 身份（API）</t>
+          <t>F. 验收（等你确认）</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t>主界面无注册入口</t>
+          <t>反馈流转</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
         <is>
-          <t>看主页面</t>
+          <t>退回后让 agent 重新 complete（或编辑改状态到等你确认）</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>页面上**没有** Agent 注册表单；agent 信息只出现在卡片/抽屉里</t>
+          <t>退回反馈被清除，新一轮验收重新开始</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
@@ -1730,7 +1730,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t>API 注册并接取</t>
+          <t>主界面无注册入口</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
         <is>
-          <t>先 `curl -F "file=@头像.png" .../api/avatars` 记 path，再 `curl -X POST -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;path&gt;"}' .../api/tasks/&lt;id&gt;/claim`</t>
+          <t>看主页面</t>
         </is>
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>返回 200，卡片移到处理中列，右上角显示头像</t>
+          <t>页面上**没有** Agent 注册表单；agent 信息只出现在卡片/抽屉里</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
@@ -1767,7 +1767,7 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>G3</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
@@ -1777,17 +1777,17 @@
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t>界面不显示 agentId</t>
+          <t>API 注册并接取</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
         <is>
-          <t>看卡片与抽屉</t>
+          <t>先 `curl -F "file=@头像.png" .../api/avatars` 记 path，再 `curl -X POST -d '{"agentId":"a1","name":"Alpha","avatar":"&lt;path&gt;"}' .../api/tasks/&lt;id&gt;/claim`</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>只显示头像 + 名称，**不显示** agentId（仅存在于 API 层）</t>
+          <t>返回 200，卡片移到处理中列，右上角显示头像</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
@@ -1804,7 +1804,7 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>G4</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
@@ -1814,17 +1814,17 @@
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t>缺名称/头像被拒</t>
+          <t>界面不显示 agentId</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
         <is>
-          <t>claim 缺 `name`、头像用字母/emoji、或伪造 `/api/avatars/xxx.png`</t>
+          <t>看卡片与抽屉</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>返回 422，任务不被接取</t>
+          <t>只显示头像 + 名称，**不显示** agentId（仅存在于 API 层）</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
@@ -1841,7 +1841,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>G5</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t>抢同一任务</t>
+          <t>缺名称/头像被拒</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
         <is>
-          <t>两个不同 agentId 先后 claim 同一任务</t>
+          <t>claim 缺 `name`、头像用字母/emoji、或伪造 `/api/avatars/xxx.png`</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="0">
         <is>
-          <t>**只有一个成功**，另一个 409</t>
+          <t>返回 422，任务不被接取</t>
         </is>
       </c>
       <c r="F49" t="inlineStr" s="0">
@@ -1878,27 +1878,27 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>H1</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
         <is>
-          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
+          <t>G. 接取任务 &amp; agent 身份（API）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t>无 agent 操作按钮</t>
+          <t>抢同一任务</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
         <is>
-          <t>看处理中/遇到阻碍列卡片与抽屉</t>
+          <t>两个不同 agentId 先后 claim 同一任务</t>
         </is>
       </c>
       <c r="E50" t="inlineStr" s="0">
         <is>
-          <t>没有「阻碍/完成/解除阻碍」按钮（这些是 agent 的 API 动作）</t>
+          <t>**只有一个成功**，另一个 409</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="0">
@@ -1915,7 +1915,7 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>H2</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t>API 状态流转</t>
+          <t>无 agent 操作按钮</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
         <is>
-          <t>curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
+          <t>看处理中/遇到阻碍列卡片与抽屉</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="0">
         <is>
-          <t>卡片在列间正确移动</t>
+          <t>没有「阻碍/完成/解除阻碍」按钮（这些是 agent 的 API 动作）</t>
         </is>
       </c>
       <c r="F51" t="inlineStr" s="0">
@@ -1952,7 +1952,7 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>H3</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t>block 带原因</t>
+          <t>API 状态流转</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -d '{"reason":"等 token"}' .../block`</t>
+          <t>curl 调 `POST /api/tasks/&lt;id&gt;/block`、`unblock`、`complete`</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="0">
         <is>
-          <t>卡片与抽屉显示该原因；unblock 后消失</t>
+          <t>卡片在列间正确移动</t>
         </is>
       </c>
       <c r="F52" t="inlineStr" s="0">
@@ -1989,27 +1989,27 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>I1</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t>I. 回收孤儿任务</t>
+          <t>H. 状态流转（agent 通过 API，界面无按钮）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t>抽屉回收</t>
+          <t>block 带原因</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
         <is>
-          <t>处理中卡片打开抽屉 →「回收到待处理」</t>
+          <t>`curl -X POST -d '{"reason":"等 token"}' .../block`</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="0">
         <is>
-          <t>卡片回到待处理列，agent 头像消失</t>
+          <t>卡片与抽屉显示该原因；unblock 后消失</t>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="0">
@@ -2026,7 +2026,7 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>I2</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t>回收后重新接取</t>
+          <t>抽屉回收</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
         <is>
-          <t>回收后由 agent 重新 claim</t>
+          <t>处理中卡片打开抽屉 →「回收到待处理」</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="0">
         <is>
-          <t>能成功接取</t>
+          <t>卡片回到待处理列，agent 头像消失</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="0">
@@ -2063,7 +2063,7 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
-          <t>I3</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="0">
@@ -2073,17 +2073,17 @@
       </c>
       <c r="C55" t="inlineStr" s="0">
         <is>
-          <t>API 回收</t>
+          <t>回收后重新接取</t>
         </is>
       </c>
       <c r="D55" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST .../api/tasks/&lt;id&gt;/recycle`</t>
+          <t>回收后由 agent 重新 claim</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="0">
         <is>
-          <t>同样回到待处理</t>
+          <t>能成功接取</t>
         </is>
       </c>
       <c r="F55" t="inlineStr" s="0">
@@ -2100,27 +2100,27 @@
     <row r="56">
       <c r="A56" t="inlineStr" s="0">
         <is>
-          <t>J1</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="0">
         <is>
-          <t>J. 归档历史</t>
+          <t>I. 回收孤儿任务</t>
         </is>
       </c>
       <c r="C56" t="inlineStr" s="0">
         <is>
-          <t>入口位置</t>
+          <t>API 回收</t>
         </is>
       </c>
       <c r="D56" t="inlineStr" s="0">
         <is>
-          <t>看顶栏</t>
+          <t>`curl -X POST .../api/tasks/&lt;id&gt;/recycle`</t>
         </is>
       </c>
       <c r="E56" t="inlineStr" s="0">
         <is>
-          <t>顶栏没有「归档历史」主按钮；在设置（齿轮）菜单里打开</t>
+          <t>同样回到待处理</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="0">
@@ -2137,7 +2137,7 @@
     <row r="57">
       <c r="A57" t="inlineStr" s="0">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="0">
@@ -2147,17 +2147,17 @@
       </c>
       <c r="C57" t="inlineStr" s="0">
         <is>
-          <t>历史详情</t>
+          <t>入口位置</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="0">
         <is>
-          <t>打开归档历史</t>
+          <t>看顶栏</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="0">
         <is>
-          <t>显示标题、workspace、标签、完成时间</t>
+          <t>顶栏没有「归档历史」主按钮；在设置（齿轮）菜单里打开</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="0">
@@ -2174,7 +2174,7 @@
     <row r="58">
       <c r="A58" t="inlineStr" s="0">
         <is>
-          <t>J3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="0">
@@ -2184,17 +2184,17 @@
       </c>
       <c r="C58" t="inlineStr" s="0">
         <is>
-          <t>单条删除</t>
+          <t>历史详情</t>
         </is>
       </c>
       <c r="D58" t="inlineStr" s="0">
         <is>
-          <t>点某条「删除」→ 确认</t>
+          <t>打开归档历史</t>
         </is>
       </c>
       <c r="E58" t="inlineStr" s="0">
         <is>
-          <t>该条消失</t>
+          <t>显示标题、workspace、标签、完成时间</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="0">
@@ -2211,7 +2211,7 @@
     <row r="59">
       <c r="A59" t="inlineStr" s="0">
         <is>
-          <t>J4</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="0">
@@ -2221,17 +2221,17 @@
       </c>
       <c r="C59" t="inlineStr" s="0">
         <is>
-          <t>全选删除</t>
+          <t>单条删除</t>
         </is>
       </c>
       <c r="D59" t="inlineStr" s="0">
         <is>
-          <t>勾选若干条（或全选）→「删除选中」→ 确认</t>
+          <t>点某条「删除」→ 确认</t>
         </is>
       </c>
       <c r="E59" t="inlineStr" s="0">
         <is>
-          <t>选中条目全部消失</t>
+          <t>该条消失</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="0">
@@ -2248,27 +2248,27 @@
     <row r="60">
       <c r="A60" t="inlineStr" s="0">
         <is>
-          <t>K1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B60" t="inlineStr" s="0">
         <is>
-          <t>K. 搜索与筛选</t>
+          <t>J. 归档历史</t>
         </is>
       </c>
       <c r="C60" t="inlineStr" s="0">
         <is>
-          <t>搜索标题</t>
+          <t>全选删除</t>
         </is>
       </c>
       <c r="D60" t="inlineStr" s="0">
         <is>
-          <t>顶栏搜索框输入标题关键词</t>
+          <t>勾选若干条（或全选）→「删除选中」→ 确认</t>
         </is>
       </c>
       <c r="E60" t="inlineStr" s="0">
         <is>
-          <t>看板就地过滤，四列结构保持</t>
+          <t>选中条目全部消失</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="0">
@@ -2285,7 +2285,7 @@
     <row r="61">
       <c r="A61" t="inlineStr" s="0">
         <is>
-          <t>K2</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr" s="0">
@@ -2295,17 +2295,17 @@
       </c>
       <c r="C61" t="inlineStr" s="0">
         <is>
-          <t>搜索 workspace</t>
+          <t>搜索标题</t>
         </is>
       </c>
       <c r="D61" t="inlineStr" s="0">
         <is>
-          <t>输入文件夹名（如 light-kanban）</t>
+          <t>顶栏搜索框输入标题关键词</t>
         </is>
       </c>
       <c r="E61" t="inlineStr" s="0">
         <is>
-          <t>该 workspace 的任务被筛出（全路径与简称都能命中）</t>
+          <t>看板就地过滤，四列结构保持</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="0">
@@ -2322,7 +2322,7 @@
     <row r="62">
       <c r="A62" t="inlineStr" s="0">
         <is>
-          <t>K3</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B62" t="inlineStr" s="0">
@@ -2332,17 +2332,17 @@
       </c>
       <c r="C62" t="inlineStr" s="0">
         <is>
-          <t>搜索 Agent</t>
+          <t>搜索 workspace</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="0">
         <is>
-          <t>输入 agent 名称</t>
+          <t>输入文件夹名（如 light-kanban）</t>
         </is>
       </c>
       <c r="E62" t="inlineStr" s="0">
         <is>
-          <t>该 agent 持有的任务被筛出</t>
+          <t>该 workspace 的任务被筛出（全路径与简称都能命中）</t>
         </is>
       </c>
       <c r="F62" t="inlineStr" s="0">
@@ -2359,7 +2359,7 @@
     <row r="63">
       <c r="A63" t="inlineStr" s="0">
         <is>
-          <t>K4</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr" s="0">
@@ -2369,17 +2369,17 @@
       </c>
       <c r="C63" t="inlineStr" s="0">
         <is>
-          <t>组合筛选</t>
+          <t>搜索 Agent</t>
         </is>
       </c>
       <c r="D63" t="inlineStr" s="0">
         <is>
-          <t>筛选里勾 Workspace=light-kanban + 标签=ui</t>
+          <t>输入 agent 名称</t>
         </is>
       </c>
       <c r="E63" t="inlineStr" s="0">
         <is>
-          <t>看板只显示同时匹配的任务，筛选按钮显示激活数量</t>
+          <t>该 agent 持有的任务被筛出</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="0">
@@ -2396,7 +2396,7 @@
     <row r="64">
       <c r="A64" t="inlineStr" s="0">
         <is>
-          <t>K5</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="B64" t="inlineStr" s="0">
@@ -2406,17 +2406,17 @@
       </c>
       <c r="C64" t="inlineStr" s="0">
         <is>
-          <t>清除筛选</t>
+          <t>组合筛选</t>
         </is>
       </c>
       <c r="D64" t="inlineStr" s="0">
         <is>
-          <t>点「清除全部」</t>
+          <t>筛选里勾 Workspace=light-kanban + 标签=ui</t>
         </is>
       </c>
       <c r="E64" t="inlineStr" s="0">
         <is>
-          <t>看板恢复完整</t>
+          <t>看板只显示同时匹配的任务，筛选按钮显示激活数量</t>
         </is>
       </c>
       <c r="F64" t="inlineStr" s="0">
@@ -2433,27 +2433,27 @@
     <row r="65">
       <c r="A65" t="inlineStr" s="0">
         <is>
-          <t>L1</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="B65" t="inlineStr" s="0">
         <is>
-          <t>L. Agent 预配置（API）</t>
+          <t>K. 搜索与筛选</t>
         </is>
       </c>
       <c r="C65" t="inlineStr" s="0">
         <is>
-          <t>预配置 agent</t>
+          <t>清除筛选</t>
         </is>
       </c>
       <c r="D65" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -d '{"id":"a1","name":"Alpha"}' .../api/agents`</t>
+          <t>点「清除全部」</t>
         </is>
       </c>
       <c r="E65" t="inlineStr" s="0">
         <is>
-          <t>成功；`curl .../api/agents` 能看到</t>
+          <t>看板恢复完整</t>
         </is>
       </c>
       <c r="F65" t="inlineStr" s="0">
@@ -2470,7 +2470,7 @@
     <row r="66">
       <c r="A66" t="inlineStr" s="0">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr" s="0">
@@ -2480,17 +2480,17 @@
       </c>
       <c r="C66" t="inlineStr" s="0">
         <is>
-          <t>更新头像</t>
+          <t>预配置 agent</t>
         </is>
       </c>
       <c r="D66" t="inlineStr" s="0">
         <is>
-          <t>上传头像后 POST /api/agents 带 `avatar`</t>
+          <t>`curl -X POST -d '{"id":"a1","name":"Alpha"}' .../api/agents`</t>
         </is>
       </c>
       <c r="E66" t="inlineStr" s="0">
         <is>
-          <t>之后该 agent 接取的卡片显示新头像</t>
+          <t>成功；`curl .../api/agents` 能看到</t>
         </is>
       </c>
       <c r="F66" t="inlineStr" s="0">
@@ -2507,7 +2507,7 @@
     <row r="67">
       <c r="A67" t="inlineStr" s="0">
         <is>
-          <t>L3</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="B67" t="inlineStr" s="0">
@@ -2517,17 +2517,17 @@
       </c>
       <c r="C67" t="inlineStr" s="0">
         <is>
-          <t>身份钉死</t>
+          <t>更新头像</t>
         </is>
       </c>
       <c r="D67" t="inlineStr" s="0">
         <is>
-          <t>预配置后该 agent claim 时带别的名称/头像</t>
+          <t>上传头像后 POST /api/agents 带 `avatar`</t>
         </is>
       </c>
       <c r="E67" t="inlineStr" s="0">
         <is>
-          <t>卡片仍显示预配置的名称和头像</t>
+          <t>之后该 agent 接取的卡片显示新头像</t>
         </is>
       </c>
       <c r="F67" t="inlineStr" s="0">
@@ -2544,27 +2544,27 @@
     <row r="68">
       <c r="A68" t="inlineStr" s="0">
         <is>
-          <t>M1</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="B68" t="inlineStr" s="0">
         <is>
-          <t>M. API 抽查（可选，用命令行）</t>
+          <t>L. Agent 预配置（API）</t>
         </is>
       </c>
       <c r="C68" t="inlineStr" s="0">
         <is>
-          <t>健康检查</t>
+          <t>身份钉死</t>
         </is>
       </c>
       <c r="D68" t="inlineStr" s="0">
         <is>
-          <t>`curl http://localhost:8641/api/health`</t>
+          <t>预配置后该 agent claim 时带别的名称/头像</t>
         </is>
       </c>
       <c r="E68" t="inlineStr" s="0">
         <is>
-          <t>`{"db":"ok","status":"ok"}`</t>
+          <t>卡片仍显示预配置的名称和头像</t>
         </is>
       </c>
       <c r="F68" t="inlineStr" s="0">
@@ -2581,7 +2581,7 @@
     <row r="69">
       <c r="A69" t="inlineStr" s="0">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr" s="0">
@@ -2591,17 +2591,17 @@
       </c>
       <c r="C69" t="inlineStr" s="0">
         <is>
-          <t>创建任务</t>
+          <t>健康检查</t>
         </is>
       </c>
       <c r="D69" t="inlineStr" s="0">
         <is>
-          <t>`curl -X POST -d '{"title":"API 测试","workspacePath":"/tmp/x"}' .../api/tasks`</t>
+          <t>`curl http://localhost:8641/api/health`</t>
         </is>
       </c>
       <c r="E69" t="inlineStr" s="0">
         <is>
-          <t>返回任务 JSON，`"status":"todo"`</t>
+          <t>`{"db":"ok","status":"ok"}`</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="0">
@@ -2618,7 +2618,7 @@
     <row r="70">
       <c r="A70" t="inlineStr" s="0">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B70" t="inlineStr" s="0">
@@ -2628,17 +2628,17 @@
       </c>
       <c r="C70" t="inlineStr" s="0">
         <is>
-          <t>接取冲突</t>
+          <t>创建任务</t>
         </is>
       </c>
       <c r="D70" t="inlineStr" s="0">
         <is>
-          <t>对同一任务连发两次 claim</t>
+          <t>`curl -X POST -d '{"title":"API 测试","workspacePath":"/tmp/x"}' .../api/tasks`</t>
         </is>
       </c>
       <c r="E70" t="inlineStr" s="0">
         <is>
-          <t>第一次 200，第二次 409</t>
+          <t>返回任务 JSON，`"status":"todo"`</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="0">
@@ -2655,7 +2655,7 @@
     <row r="71">
       <c r="A71" t="inlineStr" s="0">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B71" t="inlineStr" s="0">
@@ -2665,17 +2665,17 @@
       </c>
       <c r="C71" t="inlineStr" s="0">
         <is>
-          <t>归档历史查询</t>
+          <t>接取冲突</t>
         </is>
       </c>
       <c r="D71" t="inlineStr" s="0">
         <is>
-          <t>`curl ".../api/tasks?status=archived"`</t>
+          <t>对同一任务连发两次 claim</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="0">
         <is>
-          <t>返回已归档数组，含 `completedAt`</t>
+          <t>第一次 200，第二次 409</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="0">
@@ -2692,7 +2692,7 @@
     <row r="72">
       <c r="A72" t="inlineStr" s="0">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B72" t="inlineStr" s="0">
@@ -2702,17 +2702,17 @@
       </c>
       <c r="C72" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>归档历史查询</t>
         </is>
       </c>
       <c r="D72" t="inlineStr" s="0">
         <is>
-          <t>`curl ".../api/fs/dirs?path=%2F"`（Mac）</t>
+          <t>`curl ".../api/tasks?status=archived"`</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>返回已归档数组，含 `completedAt`</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="0">
@@ -2729,27 +2729,27 @@
     <row r="73">
       <c r="A73" t="inlineStr" s="0">
         <is>
-          <t>N1</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B73" t="inlineStr" s="0">
         <is>
-          <t>N. 跨平台（Mac）</t>
+          <t>M. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C73" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>目录浏览</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="0">
         <is>
-          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8641`</t>
+          <t>`curl ".../api/fs/dirs?path=%2F"`（Mac）</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>返回该目录下的子文件夹列表</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="0">
@@ -2766,7 +2766,7 @@
     <row r="74">
       <c r="A74" t="inlineStr" s="0">
         <is>
-          <t>N2</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr" s="0">
@@ -2776,17 +2776,17 @@
       </c>
       <c r="C74" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8641`</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="0">
@@ -2803,35 +2803,72 @@
     <row r="75">
       <c r="A75" t="inlineStr" s="0">
         <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr" s="0">
+        <is>
+          <t>N. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr" s="0">
+        <is>
           <t>N3</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr" s="0">
+      <c r="B76" t="inlineStr" s="0">
         <is>
           <t>N. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr" s="0">
+      <c r="C76" t="inlineStr" s="0">
         <is>
           <t>Gatekeeper</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr" s="0">
+      <c r="D76" t="inlineStr" s="0">
         <is>
           <t>首次运行若提示"无法验证开发者"</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr" s="0">
+      <c r="E76" t="inlineStr" s="0">
         <is>
           <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr" s="0">
+      <c r="F76" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2839,7 +2876,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F75">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F76">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: sync v1.0.3 — loopback default, status filter API, make check/CI, checklist O section
- README/README_CN: 127.0.0.1 default + LAN opt-in (-addr :8641), status
  filter values + column ordering, make check / CI, Windows firewall note
- AGENTS: pre-commit gate, dist-ships-with-source rule, cmd test seam
- PROGRESS: v1.0.3 status, fix Vite proxy port typo (:8080 -> :8641),
  mark completed v1.0.2 todos, Mac migration gains make check
- spec: exact GET /api/tasks semantics, ordering + atomic PATCH + default
  binding decisions, honest test-seam description
- manual-test-checklist: replace stale /api/fs/dirs row with fs/open+pick,
  add section O (network / API filter / PATCH atomicity); xlsx regenerated
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G89"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -2739,17 +2739,17 @@
       </c>
       <c r="C73" t="inlineStr" s="0">
         <is>
-          <t>目录浏览</t>
+          <t>打开项目文件夹</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="0">
         <is>
-          <t>`curl ".../api/fs/dirs?path=%2F"`（Mac）</t>
+          <t>`curl -X POST -d '{"path":"/tmp"}' .../api/fs/open`</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="0">
         <is>
-          <t>返回该目录下的子文件夹列表</t>
+          <t>服务器系统文件管理器打开该文件夹，返回 `{"ok":"true"}`</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="0">
@@ -2766,27 +2766,27 @@
     <row r="74">
       <c r="A74" t="inlineStr" s="0">
         <is>
-          <t>N1</t>
+          <t>M5b</t>
         </is>
       </c>
       <c r="B74" t="inlineStr" s="0">
         <is>
-          <t>N. 跨平台（Mac）</t>
+          <t>M. API 抽查（可选，用命令行）</t>
         </is>
       </c>
       <c r="C74" t="inlineStr" s="0">
         <is>
-          <t>Apple Silicon</t>
+          <t>系统文件夹选择器</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="0">
         <is>
-          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8641`</t>
+          <t>`curl -X POST .../api/fs/pick`（仅桌面环境）</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>弹出系统文件夹窗口：选择后返回 `{"path":"/..."}`，取消返回 `{"path":""}`</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="0">
@@ -2803,7 +2803,7 @@
     <row r="75">
       <c r="A75" t="inlineStr" s="0">
         <is>
-          <t>N2</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr" s="0">
@@ -2813,17 +2813,17 @@
       </c>
       <c r="C75" t="inlineStr" s="0">
         <is>
-          <t>Intel Mac</t>
+          <t>Apple Silicon</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="0">
         <is>
-          <t>用 `dist/light-kanban-darwin-amd64`</t>
+          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8641`</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="0">
         <is>
-          <t>同上</t>
+          <t>正常启动，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="0">
@@ -2840,35 +2840,516 @@
     <row r="76">
       <c r="A76" t="inlineStr" s="0">
         <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr" s="0">
+        <is>
+          <t>N. 跨平台（Mac）</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr" s="0">
+        <is>
+          <t>Intel Mac</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr" s="0">
+        <is>
+          <t>用 `dist/light-kanban-darwin-amd64`</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr" s="0">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr" s="0">
+        <is>
           <t>N3</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr" s="0">
+      <c r="B77" t="inlineStr" s="0">
         <is>
           <t>N. 跨平台（Mac）</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr" s="0">
+      <c r="C77" t="inlineStr" s="0">
         <is>
           <t>Gatekeeper</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr" s="0">
+      <c r="D77" t="inlineStr" s="0">
         <is>
           <t>首次运行若提示"无法验证开发者"</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr" s="0">
+      <c r="E77" t="inlineStr" s="0">
         <is>
           <t>右键 → 打开，或 `xattr -dr com.apple.quarantine ./light-kanban-darwin-arm64` 后重试</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr" s="0">
+      <c r="F77" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr" s="0">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr" s="0">
+        <is>
+          <t>默认仅本机监听</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr" s="0">
+        <is>
+          <t>直接 `./dist/light-kanban`（不带 `-addr`）</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr" s="0">
+        <is>
+          <t>`curl http://127.0.0.1:8641/api/health` 返回 ok；用本机局域网 IP（`curl http://&lt;LAN-IP&gt;:8641/api/health`）或另一台电脑访问连不上</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr" s="0">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr" s="0">
+        <is>
+          <t>显式 LAN 模式</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr" s="0">
+        <is>
+          <t>`./dist/light-kanban -addr :8641`</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr" s="0">
+        <is>
+          <t>局域网内另一台电脑能打开 http://&lt;主机LAN-IP&gt;:8641</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr" s="0">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="0">
+        <is>
+          <t>启动自动开浏览器</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr" s="0">
+        <is>
+          <t>默认启动（不带 `-no-open`）</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr" s="0">
+        <is>
+          <t>浏览器自动打开 http://127.0.0.1:8641</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr" s="0">
+        <is>
+          <t>O4</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="0">
+        <is>
+          <t>待处理过滤</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr" s="0">
+        <is>
+          <t>灌几条不同状态任务后 `curl ".../api/tasks?status=todo"`</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr" s="0">
+        <is>
+          <t>只返回待处理任务</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr" s="0">
+        <is>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="0">
+        <is>
+          <t>处理中过滤</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr" s="0">
+        <is>
+          <t>`curl ".../api/tasks?status=in_progress"`</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr" s="0">
+        <is>
+          <t>只返回处理中任务</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr" s="0">
+        <is>
+          <t>O6</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr" s="0">
+        <is>
+          <t>遇到阻碍过滤</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr" s="0">
+        <is>
+          <t>`curl ".../api/tasks?status=blocked"`</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr" s="0">
+        <is>
+          <t>只返回遇到阻碍任务</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr" s="0">
+        <is>
+          <t>O7</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr" s="0">
+        <is>
+          <t>等你确认过滤</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr" s="0">
+        <is>
+          <t>`curl ".../api/tasks?status=awaiting_confirmation"`</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr" s="0">
+        <is>
+          <t>只返回等你确认任务</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr" s="0">
+        <is>
+          <t>O8</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="0">
+        <is>
+          <t>active 与非法值</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr" s="0">
+        <is>
+          <t>`curl ".../api/tasks?status=active"` 与 `?status=banana`</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr" s="0">
+        <is>
+          <t>active 等同无过滤；banana 返回 400</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr" s="0">
+        <is>
+          <t>O9</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="0">
+        <is>
+          <t>待处理 FIFO</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr" s="0">
+        <is>
+          <t>先后创建两个待处理任务，再查 `?status=todo`</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr" s="0">
+        <is>
+          <t>先创建的任务排在前面（最老在前）</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr" s="0">
+        <is>
+          <t>O10</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr" s="0">
+        <is>
+          <t>PATCH 一次修改</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr" s="0">
+        <is>
+          <t>`curl -X PATCH -d '{"title":"新标题","status":"blocked"}' .../api/tasks/&lt;id&gt;`</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr" s="0">
+        <is>
+          <t>返回 200，标题与状态同时生效</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr" s="0">
+        <is>
+          <t>O11</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr" s="0">
+        <is>
+          <t>PATCH 非法状态无残留</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr" s="0">
+        <is>
+          <t>`curl -X PATCH -d '{"title":"不应保存","status":"banana"}' .../api/tasks/&lt;id&gt;`</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr" s="0">
+        <is>
+          <t>返回 422；再 GET 该任务，标题仍是修改前的值</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr" s="0">
+        <is>
+          <t>O12</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr" s="0">
+        <is>
+          <t>O. v1.0.3 加固（网络 / API 过滤 / PATCH 原子性）</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="0">
+        <is>
+          <t>归档排序</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr" s="0">
+        <is>
+          <t>先后归档两条任务后查 `?status=archived`</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr" s="0">
+        <is>
+          <t>最近完成的那条排在最上面</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -2876,7 +3357,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F76">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F89">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore: finish v1.0.3 post-release housekeeping
- make run now inherits the loopback-only default (127.0.0.1:8641) instead
  of forcing -addr :8641; make run-lan is the explicit LAN variant
- README/README_CN run-from-source examples drop -addr :8641 from the
  default flow (LAN stays an explicit, separately-labelled opt-in)
- manual checklist baseline is now default mode: preamble, A1/A1b/A2/A3
  and N1 run without -addr at http://127.0.0.1:8641; LAN testing lives
  only in section O; xlsx regenerated
- PROGRESS: latest release = v1.0.3 (released), no pending release todo,
  stable-maintenance state
- frontend package metadata bumped to 1.0.3 (package.json + lock root
  version only; zero functional frontend diff, embedded dist unchanged)
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -117,12 +117,12 @@
       </c>
       <c r="D2" t="inlineStr" s="0">
         <is>
-          <t>运行 `./dist/light-kanban -addr :8641`</t>
+          <t>运行 `./dist/light-kanban`（默认，不加 `-addr`）</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>命令行出现 `listening on :8641`，不报错</t>
+          <t>命令行出现 `listening on 127.0.0.1:8641`，不报错；本机打开 http://127.0.0.1:8641 正常</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -159,7 +159,7 @@
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>弹出控制台窗口并**自动打开浏览器** http://localhost:8641</t>
+          <t>弹出控制台窗口并**自动打开浏览器** http://127.0.0.1:8641</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
@@ -191,7 +191,7 @@
       </c>
       <c r="D4" t="inlineStr" s="0">
         <is>
-          <t>浏览器开 http://localhost:8641/api/health</t>
+          <t>浏览器开 http://127.0.0.1:8641/api/health</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="0">
@@ -228,7 +228,7 @@
       </c>
       <c r="D5" t="inlineStr" s="0">
         <is>
-          <t>打开 http://localhost:8641</t>
+          <t>打开 http://127.0.0.1:8641</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="0">
@@ -2818,12 +2818,12 @@
       </c>
       <c r="D75" t="inlineStr" s="0">
         <is>
-          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64 -addr :8641`</t>
+          <t>`chmod +x` 后运行 `./light-kanban-darwin-arm64`（默认模式）</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="0">
         <is>
-          <t>正常启动，页面功能同 Windows</t>
+          <t>正常启动，监听 127.0.0.1:8641，页面功能同 Windows</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="0">

</xml_diff>

<commit_message>
feat: v1.0.4 — archive open-folder shortcut + interactive product tour
- Archive history rows get a folder icon (same openFolder API, icon and
  error handling as the task drawer); delete / select-all unchanged
- Replace the centered wizard modal with an interactive product tour that
  runs on the real UI: stable data-tour targets, dimmed click-blocked
  overlay with cutouts, auto-placed coachmark, real clicks/typing advance,
  created-task tracking via data-tour-task-id, optional-step skip and
  bounded missing-target recovery (no infinite waits)
- Persistence: only Finish writes lk-tour-v1-completed=1; Skip/Esc/reload
  never mark completion; Settings -> Guide replays without clearing it
- Tour decision logic extracted as pure DOM-free functions
  (components/ProductTour/logic.ts + steps.ts) with 37 vitest cases wired
  into make check and CI; frontend package metadata bumped to 1.0.4
- Docs synced: README/README_CN, PROGRESS, spec, manual checklist + xlsx
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G115"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -302,12 +302,12 @@
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>新开无痕窗口（或清掉 localStorage `lk-wizard-seen`）打开页面</t>
+          <t>新开无痕窗口（或清掉 localStorage `lk-tour-v1-completed`）打开页面</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t>自动弹出 4 步引导向导，可上一步 / 下一步 / 跳过</t>
+          <t>自动在**真实界面**上启动交互式产品导览（遮罩暗化 + 目标高亮 + coachmark），不是旧的居中向导弹窗；细节见 Q 节</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
@@ -381,7 +381,7 @@
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>整个界面（列名、按钮、弹窗、抽屉、向导）在中英文间即时切换；刷新后保持</t>
+          <t>整个界面（列名、按钮、弹窗、抽屉、导览）在中英文间即时切换；刷新后保持</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
@@ -413,12 +413,12 @@
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t>点「跳过」或「开始使用」后刷新页面</t>
+          <t>完整走完导览点「完成」后刷新页面</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>刷新后不再自动弹出</t>
+          <t>刷新后不再自动弹出；如果只是「跳过」，刷新后仍会再次自动出现</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
@@ -3355,9 +3355,971 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr" s="0">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr" s="0">
+        <is>
+          <t>P. v1.0.4 归档历史打开目录</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="0">
+        <is>
+          <t>文件夹图标</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr" s="0">
+        <is>
+          <t>打开 设置 → 归档历史</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr" s="0">
+        <is>
+          <t>每条记录的「完成于」下方显示 文件夹图标 + 删除按钮，样式与任务抽屉里的文件夹图标一致，行高不变</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr" s="0">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr" s="0">
+        <is>
+          <t>P. v1.0.4 归档历史打开目录</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr" s="0">
+        <is>
+          <t>打开项目目录</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr" s="0">
+        <is>
+          <t>点某条记录的文件夹图标</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr" s="0">
+        <is>
+          <t>服务器那台电脑的文件管理器打开并定位到该 workspace 目录；Archive Dialog 不关闭，归档状态不变</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr" s="0">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr" s="0">
+        <is>
+          <t>P. v1.0.4 归档历史打开目录</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="0">
+        <is>
+          <t>路径不存在/打开失败</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr" s="0">
+        <is>
+          <t>找一条 workspacePath 已不存在（如已删除目录）的记录点文件夹图标</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr" s="0">
+        <is>
+          <t>弹出与任务抽屉一致的错误提示（alert 操作失败），不影响其他功能</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr" s="0">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr" s="0">
+        <is>
+          <t>P. v1.0.4 归档历史打开目录</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="0">
+        <is>
+          <t>删除仍正常</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr" s="0">
+        <is>
+          <t>点「删除」→ 确认；再勾选多条 →「删除选中」→ 确认</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr" s="0">
+        <is>
+          <t>单条 / 批量删除都正常，选中态正确</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr" s="0">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr" s="0">
+        <is>
+          <t>P. v1.0.4 归档历史打开目录</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="0">
+        <is>
+          <t>语言切换</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr" s="0">
+        <is>
+          <t>切到 English 看归档历史</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr" s="0">
+        <is>
+          <t>文件夹图标悬停显示 "Open project folder"，其余文案为英文</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr" s="0">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="0">
+        <is>
+          <t>自动启动</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr" s="0">
+        <is>
+          <t>清 key 后刷新</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr" s="0">
+        <is>
+          <t>导览自动启动：页面其余区域暗化，**没有**旧式居中向导 Modal，第一个箭头/高亮指向顶栏「+」</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr" s="0">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="0">
+        <is>
+          <t>只允许目标操作</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr" s="0">
+        <is>
+          <t>尝试点击遮罩区域的其他按钮（搜索框、列头等）</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr" s="0">
+        <is>
+          <t>点不动；只有高亮目标（+）可点，coachmark 上的跳过可点</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr" s="0">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr" s="0">
+        <is>
+          <t>真实打开弹窗</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr" s="0">
+        <is>
+          <t>点「+」</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr" s="0">
+        <is>
+          <t>Create Task Dialog 真实打开；导览自动移动到 workspace 路径输入行，暗化遮罩在弹窗区域开洞</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr" s="0">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="0">
+        <is>
+          <t>手动输入路径</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr" s="0">
+        <is>
+          <t>在路径框输入一个存在的绝对路径</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr" s="0">
+        <is>
+          <t>输入正常；输入完成后导览自动移动到「标题」输入框</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr" s="0">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="0">
+        <is>
+          <t>选择目录</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr" s="0">
+        <is>
+          <t>回到路径框场景，点「选择…」</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr" s="0">
+        <is>
+          <t>系统文件夹窗口正常弹出并回填路径（或在无桌面环境提示失败并可继续手输）；回填后导览同样前进</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr" s="0">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr" s="0">
+        <is>
+          <t>标题</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr" s="0">
+        <is>
+          <t>输入标题</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr" s="0">
+        <is>
+          <t>输入正常；输入完成后导览移动到「创建」按钮</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr" s="0">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr" s="0">
+        <is>
+          <t>真实创建</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr" s="0">
+        <is>
+          <t>点「创建」</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr" s="0">
+        <is>
+          <t>任务真实创建、弹窗关闭；导览等待并**精确**高亮刚创建的那张卡（而不是待处理列第一张）</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr" s="0">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr" s="0">
+        <is>
+          <t>打开抽屉</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr" s="0">
+        <is>
+          <t>点刚创建的卡片</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr" s="0">
+        <is>
+          <t>Task Drawer 真实打开；导览跟随进入抽屉（高亮抽屉区域，含「任务详情」说明与下一步）</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr" s="0">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr" s="0">
+        <is>
+          <t>抽屉内控件</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr" s="0">
+        <is>
+          <t>按导览走：打开项目目录（说明步）→ 状态区（Agent 工作流说明）</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr" s="0">
+        <is>
+          <t>抽屉内文件夹图标、状态区都能被正确高亮；文件夹图标仍可真实点击</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr" s="0">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr" s="0">
+        <is>
+          <t>自动关抽屉</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr" s="0">
+        <is>
+          <t>在状态区说明步点「下一步」</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr" s="0">
+        <is>
+          <t>抽屉自动关闭，导览指向「等你确认」列头（窄窗口时自动横向滚动到该列）</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr" s="0">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr" s="0">
+        <is>
+          <t>设置与归档</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr" s="0">
+        <is>
+          <t>继续：点设置齿轮 → 点「归档历史」</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr" s="0">
+        <is>
+          <t>设置菜单真实打开；点归档后 Archive Dialog 真实打开，导览进入</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr" s="0">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr" s="0">
+        <is>
+          <t>空归档不卡死</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr" s="0">
+        <is>
+          <t>归档为空时走导览</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr" s="0">
+        <is>
+          <t>归档说明步正常显示；文件夹图标步自动跳过，不卡死，直接到完成卡</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr" s="0">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr" s="0">
+        <is>
+          <t>有归档数据</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr" s="0">
+        <is>
+          <t>有归档任务时走导览</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr" s="0">
+        <is>
+          <t>导览能定位到归档记录的文件夹图标并显示说明，可点「下一步」继续</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr" s="0">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr" s="0">
+        <is>
+          <t>Finish</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr" s="0">
+        <is>
+          <t>最后点「完成」</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr" s="0">
+        <is>
+          <t>导览关闭；localStorage 里 `lk-tour-v1-completed=1`；刷新页面导览不再自动出现</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr" s="0">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr" s="0">
+        <is>
+          <t>Q. v1.0.4 交互式产品导览（首次运行）</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr" s="0">
+        <is>
+          <t>手动重放</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr" s="0">
+        <is>
+          <t>设置 → Guide（使用向导）</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr" s="0">
+        <is>
+          <t>导览从头重新运行；结束后 completed 仍为 1</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr" s="0">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr" s="0">
+        <is>
+          <t>R. v1.0.4 导览 Skip / 恢复 / 响应式</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr" s="0">
+        <is>
+          <t>Skip 不写完成</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr" s="0">
+        <is>
+          <t>第一步点「跳过」</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr" s="0">
+        <is>
+          <t>导览关闭，`lk-tour-v1-completed` 不存在；刷新后导览再次自动出现</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr" s="0">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr" s="0">
+        <is>
+          <t>R. v1.0.4 导览 Skip / 恢复 / 响应式</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr" s="0">
+        <is>
+          <t>Esc / 中途退出</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr" s="0">
+        <is>
+          <t>导览中途按 Esc 或刷新页面</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr" s="0">
+        <is>
+          <t>导览退出且不写 completed；下次启动重新出现</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr" s="0">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr" s="0">
+        <is>
+          <t>R. v1.0.4 导览 Skip / 恢复 / 响应式</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr" s="0">
+        <is>
+          <t>目标缺失恢复</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr" s="0">
+        <is>
+          <t>在「创建」步骤点「取消」关闭弹窗</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr" s="0">
+        <is>
+          <t>约 4 秒内导览自动回到第一步指向「+」，不无限等待</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr" s="0">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr" s="0">
+        <is>
+          <t>R. v1.0.4 导览 Skip / 恢复 / 响应式</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr" s="0">
+        <is>
+          <t>核心步骤缺失提示</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr" s="0">
+        <is>
+          <t>（可选）在任务卡步骤用控制台移除目标元素</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr" s="0">
+        <is>
+          <t>超时后出现「没有找到目标控件」提示卡，可点「下一步」或「跳过」，不卡死</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr" s="0">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr" s="0">
+        <is>
+          <t>R. v1.0.4 导览 Skip / 恢复 / 响应式</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr" s="0">
+        <is>
+          <t>1440px / 1024px / 窄窗口</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr" s="0">
+        <is>
+          <t>三种窗口宽度各走一遍导览</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr" s="0">
+        <is>
+          <t>箭头不跑出屏幕；tooltip 始终在视口内；横向滚动后定位正确；抽屉/弹窗打开后定位正确</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr" s="0">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr" s="0">
+        <is>
+          <t>R. v1.0.4 导览 Skip / 恢复 / 响应式</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr" s="0">
+        <is>
+          <t>中英文</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr" s="0">
+        <is>
+          <t>中文与 English 各走一遍导览</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr" s="0">
+        <is>
+          <t>所有 coachmark 文案为对应语言，无中英混杂</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F89">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F115">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: tour gray-screen on dialog cancel + strict target-only clicking
- Root cause: the missing-target timer re-armed inside the
  MutationObserver/render loop and instantly undid the recovery state
  (setMissing(false) right after setMissing(true)), leaving the screen
  permanently dimmed. Extract a one-shot createMissingWatcher with a fired
  guard (pure, 5 new vitest cases) and wire the component through it
- Per user feedback, every step is now strictly target-only clickable: the
  widened dialog cutouts are removed, so Cancel can no longer be clicked
  mid-create-flow (Esc still exits the tour without completion); closing
  the drawer or archive dialog mid-tour loops back to the task-card /
  archive-menu step instead of dead-ending
- Docs: spec.md / PROGRESS / manual checklist (Q2, R3) + xlsx regenerated
- Verified headlessly in real Chrome: cancel blocked, dialog stays open,
  drawer-close recovers to the task-card step after ~4s
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -3595,12 +3595,12 @@
       </c>
       <c r="D96" t="inlineStr" s="0">
         <is>
-          <t>尝试点击遮罩区域的其他按钮（搜索框、列头等）</t>
+          <t>尝试点击遮罩区域的其他按钮（搜索框、列头、弹窗里的「取消」等）</t>
         </is>
       </c>
       <c r="E96" t="inlineStr" s="0">
         <is>
-          <t>点不动；只有高亮目标（+）可点，coachmark 上的跳过可点</t>
+          <t>点不动；只有高亮目标可点，coachmark 上的跳过可点；弹窗不会被意外关闭，不会灰屏</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="0">
@@ -4187,12 +4187,12 @@
       </c>
       <c r="D112" t="inlineStr" s="0">
         <is>
-          <t>在「创建」步骤点「取消」关闭弹窗</t>
+          <t>抽屉步骤点抽屉右上 × 关闭抽屉（× 在高亮区域内）</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="0">
         <is>
-          <t>约 4 秒内导览自动回到第一步指向「+」，不无限等待</t>
+          <t>约 4 秒内导览自动回到「任务卡」步骤继续，不灰屏不卡死</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="0">

</xml_diff>

<commit_message>
docs: v1.0.5 candidate — Worker Skill Quick Start, Use Cases, integration docs
README/README_CN Quick Start rewritten as the five-step released-binary +
light-kanban-worker Skill path with a copyable scheduler prompt and a
one-shot manual run example; Use Cases added (scheduled coding agent,
multi-agent queue, review loop, blocked work, cross-project queue,
boundary); raw curl demoted to Manual Agent Integration. spec.md records
the v1.0.5 no-API-change Worker Integration decisions; manual checklist
gains section S (worker integration) with regenerated xlsx; frontend
version bumped to 1.0.5; PROGRESS records the v1.0.5 candidate and its
release gate. make check and make cross (4 platforms) PASS.
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G123"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -4317,9 +4317,305 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr" s="0">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr" s="0">
+        <is>
+          <t>安装 Worker Skill</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr" s="0">
+        <is>
+          <t>`npx skills add LightDevCoder/skills#v0.1.4 --skill light-kanban-worker --yes --copy --agent '*'`</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr" s="0">
+        <is>
+          <t>安装成功；`npx --yes skills list` 列出 `light-kanban-worker`（不依赖源码 checkout）</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr" s="0">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr" s="0">
+        <is>
+          <t>一次性手动运行</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr" s="0">
+        <is>
+          <t>建一张 todo 卡后，用 prompt「Use light-kanban-worker to process one task from http://127.0.0.1:8641 as agent codex-main.」跑一次</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr" s="0">
+        <is>
+          <t>Agent 领取该卡 → 进入 workspace 执行 → `complete` → 卡片到**等你确认**，本次运行结束</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr" s="0">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr" s="0">
+        <is>
+          <t>定时 prompt</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr" s="0">
+        <is>
+          <t>用 README Quick Start 第四步的 scheduler prompt 创建每 15 分钟（或更短）的定时任务</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr" s="0">
+        <is>
+          <t>每次唤醒只处理一张卡；没有卡时正常结束，不新建任务、不卡死</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr" s="0">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr" s="0">
+        <is>
+          <t>退回修改闭环</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr" s="0">
+        <is>
+          <t>对**等你确认**卡点「退回修改」并附反馈</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr" s="0">
+        <is>
+          <t>下一次唤醒同一 Agent 优先处理该卡，按反馈修改后重新 `complete` 到**等你确认**；不需要新建任务</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr" s="0">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr" s="0">
+        <is>
+          <t>workspace 缺失</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr" s="0">
+        <is>
+          <t>新建一张 workspace 路径不存在的卡</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr" s="0">
+        <is>
+          <t>Worker 领取后 block，卡上显示「Workspace path is not accessible from this agent host.」</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr" s="0">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr" s="0">
+        <is>
+          <t>双 Agent 原子领取</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr" s="0">
+        <is>
+          <t>两个不同 agentId 同时领取同一张 todo（或手动并发两次 claim）</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr" s="0">
+        <is>
+          <t>恰好一个 200、一个 409；输家重读队列后结束，不会死循环</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr" s="0">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr" s="0">
+        <is>
+          <t>空队列</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr" s="0">
+        <is>
+          <t>清空所有活跃任务后运行一次 worker</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr" s="0">
+        <is>
+          <t>「No task available」干净退出；数据库无变化</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr" s="0">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr" s="0">
+        <is>
+          <t>服务离线</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr" s="0">
+        <is>
+          <t>停掉 Light-Kanban 后运行一次 worker</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr" s="0">
+        <is>
+          <t>清晰报错结束；不修改任何任务</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F115">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F123">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: vendor light-kanban-worker Skill snapshot for offline/manual install
skills/light-kanban-worker/ is a byte-identical snapshot of
LightDevCoder/skills v0.1.4 (commit a9cc8aa). skills/manifest.json pins
source identity and per-file SHA-256; scripts/verify-vendored-skill.cjs
(with positive/negative self-test) is wired into make check and CI so the
snapshot cannot drift. README Quick Start Step 2 now offers both install
paths (npx recommended, manual copy offline); AGENTS.md, spec.md,
PROGRESS.md, and the manual checklist (S1b + regenerated xlsx) updated.
</commit_message>
<xml_diff>
--- a/docs/light-kanban-验收清单.xlsx
+++ b/docs/light-kanban-验收清单.xlsx
@@ -51,7 +51,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -4357,7 +4357,7 @@
     <row r="117">
       <c r="A117" t="inlineStr" s="0">
         <is>
-          <t>S2</t>
+          <t>S1b</t>
         </is>
       </c>
       <c r="B117" t="inlineStr" s="0">
@@ -4367,17 +4367,17 @@
       </c>
       <c r="C117" t="inlineStr" s="0">
         <is>
-          <t>一次性手动运行</t>
+          <t>手动复制安装（离线 / 无 npx）</t>
         </is>
       </c>
       <c r="D117" t="inlineStr" s="0">
         <is>
-          <t>建一张 todo 卡后，用 prompt「Use light-kanban-worker to process one task from http://127.0.0.1:8641 as agent codex-main.」跑一次</t>
+          <t>把本仓库 `skills/light-kanban-worker/` 整个目录复制到 host 认可的 skills root（如 `~/.agents/skills/light-kanban-worker`），刷新 host</t>
         </is>
       </c>
       <c r="E117" t="inlineStr" s="0">
         <is>
-          <t>Agent 领取该卡 → 进入 workspace 执行 → `complete` → 卡片到**等你确认**，本次运行结束</t>
+          <t>host 的 skill 列表能发现 `light-kanban-worker`；`node scripts/verify-vendored-skill.cjs` 输出 `VENDOR_SKILL=PASS (10 files …)`</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="0">
@@ -4394,7 +4394,7 @@
     <row r="118">
       <c r="A118" t="inlineStr" s="0">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B118" t="inlineStr" s="0">
@@ -4404,17 +4404,17 @@
       </c>
       <c r="C118" t="inlineStr" s="0">
         <is>
-          <t>定时 prompt</t>
+          <t>一次性手动运行</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="0">
         <is>
-          <t>用 README Quick Start 第四步的 scheduler prompt 创建每 15 分钟（或更短）的定时任务</t>
+          <t>建一张 todo 卡后，用 prompt「Use light-kanban-worker to process one task from http://127.0.0.1:8641 as agent codex-main.」跑一次</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="0">
         <is>
-          <t>每次唤醒只处理一张卡；没有卡时正常结束，不新建任务、不卡死</t>
+          <t>Agent 领取该卡 → 进入 workspace 执行 → `complete` → 卡片到**等你确认**，本次运行结束</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="0">
@@ -4431,7 +4431,7 @@
     <row r="119">
       <c r="A119" t="inlineStr" s="0">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B119" t="inlineStr" s="0">
@@ -4441,17 +4441,17 @@
       </c>
       <c r="C119" t="inlineStr" s="0">
         <is>
-          <t>退回修改闭环</t>
+          <t>定时 prompt</t>
         </is>
       </c>
       <c r="D119" t="inlineStr" s="0">
         <is>
-          <t>对**等你确认**卡点「退回修改」并附反馈</t>
+          <t>用 README Quick Start 第四步的 scheduler prompt 创建每 15 分钟（或更短）的定时任务</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="0">
         <is>
-          <t>下一次唤醒同一 Agent 优先处理该卡，按反馈修改后重新 `complete` 到**等你确认**；不需要新建任务</t>
+          <t>每次唤醒只处理一张卡；没有卡时正常结束，不新建任务、不卡死</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="0">
@@ -4468,7 +4468,7 @@
     <row r="120">
       <c r="A120" t="inlineStr" s="0">
         <is>
-          <t>S5</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B120" t="inlineStr" s="0">
@@ -4478,17 +4478,17 @@
       </c>
       <c r="C120" t="inlineStr" s="0">
         <is>
-          <t>workspace 缺失</t>
+          <t>退回修改闭环</t>
         </is>
       </c>
       <c r="D120" t="inlineStr" s="0">
         <is>
-          <t>新建一张 workspace 路径不存在的卡</t>
+          <t>对**等你确认**卡点「退回修改」并附反馈</t>
         </is>
       </c>
       <c r="E120" t="inlineStr" s="0">
         <is>
-          <t>Worker 领取后 block，卡上显示「Workspace path is not accessible from this agent host.」</t>
+          <t>下一次唤醒同一 Agent 优先处理该卡，按反馈修改后重新 `complete` 到**等你确认**；不需要新建任务</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="0">
@@ -4505,7 +4505,7 @@
     <row r="121">
       <c r="A121" t="inlineStr" s="0">
         <is>
-          <t>S6</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="B121" t="inlineStr" s="0">
@@ -4515,17 +4515,17 @@
       </c>
       <c r="C121" t="inlineStr" s="0">
         <is>
-          <t>双 Agent 原子领取</t>
+          <t>workspace 缺失</t>
         </is>
       </c>
       <c r="D121" t="inlineStr" s="0">
         <is>
-          <t>两个不同 agentId 同时领取同一张 todo（或手动并发两次 claim）</t>
+          <t>新建一张 workspace 路径不存在的卡</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="0">
         <is>
-          <t>恰好一个 200、一个 409；输家重读队列后结束，不会死循环</t>
+          <t>Worker 领取后 block，卡上显示「Workspace path is not accessible from this agent host.」</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="0">
@@ -4542,7 +4542,7 @@
     <row r="122">
       <c r="A122" t="inlineStr" s="0">
         <is>
-          <t>S7</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="B122" t="inlineStr" s="0">
@@ -4552,17 +4552,17 @@
       </c>
       <c r="C122" t="inlineStr" s="0">
         <is>
-          <t>空队列</t>
+          <t>双 Agent 原子领取</t>
         </is>
       </c>
       <c r="D122" t="inlineStr" s="0">
         <is>
-          <t>清空所有活跃任务后运行一次 worker</t>
+          <t>两个不同 agentId 同时领取同一张 todo（或手动并发两次 claim）</t>
         </is>
       </c>
       <c r="E122" t="inlineStr" s="0">
         <is>
-          <t>「No task available」干净退出；数据库无变化</t>
+          <t>恰好一个 200、一个 409；输家重读队列后结束，不会死循环</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="0">
@@ -4579,35 +4579,72 @@
     <row r="123">
       <c r="A123" t="inlineStr" s="0">
         <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr" s="0">
+        <is>
+          <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr" s="0">
+        <is>
+          <t>空队列</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr" s="0">
+        <is>
+          <t>清空所有活跃任务后运行一次 worker</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr" s="0">
+        <is>
+          <t>「No task available」干净退出；数据库无变化</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr" s="0">
+        <is>
           <t>S8</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr" s="0">
+      <c r="B124" t="inlineStr" s="0">
         <is>
           <t>S. v1.0.5 Worker Skill 集成（scheduled worker）</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr" s="0">
+      <c r="C124" t="inlineStr" s="0">
         <is>
           <t>服务离线</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr" s="0">
+      <c r="D124" t="inlineStr" s="0">
         <is>
           <t>停掉 Light-Kanban 后运行一次 worker</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr" s="0">
+      <c r="E124" t="inlineStr" s="0">
         <is>
           <t>清晰报错结束；不修改任何任务</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr" s="0">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr" s="0">
+      <c r="F124" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr" s="0">
         <is>
           <t/>
         </is>
@@ -4615,7 +4652,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F123">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F124">
       <formula1>"✅ 通过,❌ 失败,⚠ 存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>